<commit_message>
fix & feat: Se añade instructivo para configuracion empresas y se ajustan los instructivos y plantilla de cargue de excel
</commit_message>
<xml_diff>
--- a/Assets/Plantillas/InstructivoPlantillaCargue.xlsx
+++ b/Assets/Plantillas/InstructivoPlantillaCargue.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr codeName="ThisWorkbook" hidePivotFieldList="1" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\omara\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/72c68232ab824a52/Omar Akon Personal/Proyectos OAG/Bufins Web/Common/Adicionales/Plantilla cargue/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{028B1B36-2557-4057-A3FA-7676B7B3B9C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="47" documentId="13_ncr:1_{028B1B36-2557-4057-A3FA-7676B7B3B9C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F915F77B-D69B-4721-8526-704C91356302}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="598" xr2:uid="{FA4E9C0C-F0DD-43A6-9F82-B69A727F5A7D}"/>
   </bookViews>
@@ -111,7 +111,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="57">
   <si>
     <t>GASTOS FIJOS</t>
   </si>
@@ -120,27 +120,6 @@
   </si>
   <si>
     <t>OTROS GASTOS</t>
-  </si>
-  <si>
-    <t>Ebitda</t>
-  </si>
-  <si>
-    <t>No Ebitda</t>
-  </si>
-  <si>
-    <t>ACTIVO CORRIENTE</t>
-  </si>
-  <si>
-    <t>ACTIVO NO CORRIENTE</t>
-  </si>
-  <si>
-    <t>PASIVO NO CORRIENTE</t>
-  </si>
-  <si>
-    <t>PASIVO CORRIENTE</t>
-  </si>
-  <si>
-    <t>UNIDADES</t>
   </si>
   <si>
     <t>Las hojas de este libro tiene nombres que no pueden ser cambiados</t>
@@ -161,27 +140,6 @@
     <t>Ninguna de las hojas de este libro se puede eliminar, ni ocultar</t>
   </si>
   <si>
-    <t>Z_AñoEjecucion</t>
-  </si>
-  <si>
-    <t>Z_Empresas</t>
-  </si>
-  <si>
-    <t>Z_Paises</t>
-  </si>
-  <si>
-    <t>Z_SignoCreditos</t>
-  </si>
-  <si>
-    <t>Z_Categorias</t>
-  </si>
-  <si>
-    <t>Z_Moneda</t>
-  </si>
-  <si>
-    <t>Z_Unidades</t>
-  </si>
-  <si>
     <t>Z_BalancePrueba</t>
   </si>
   <si>
@@ -195,27 +153,6 @@
   </si>
   <si>
     <t>Z_TablaPUC</t>
-  </si>
-  <si>
-    <t>Coloque el año actual sin puntos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Coloque el nombre de las empresas a consolidar. Estos nombres deberán ser siempre idénticos a la forma en que se reportarán en las bases de datos. </t>
-  </si>
-  <si>
-    <t>Si las cuentas de pasivo, patrimonio e ingresos se reportan con signo negativo coloque acá el signo menos</t>
-  </si>
-  <si>
-    <t>En la columna K de la hoja de Z_CteYnoCte se disciminan los activos y pasivos por corrientes y no corrientes, tenga en cuenta que la descipción correcta para cada rubro es la que se indica en esta lista:</t>
-  </si>
-  <si>
-    <t>Indique el fomato de los datos. Estos deben ser:</t>
-  </si>
-  <si>
-    <t>MILES</t>
-  </si>
-  <si>
-    <t>MILLONES</t>
   </si>
   <si>
     <t>El nombre de las empresas deberá estar escrito en forma idéntica a como se reportó en la hoja de Z_Empresa</t>
@@ -234,24 +171,6 @@
   </si>
   <si>
     <t>En la celda A1 coloque los datos del balance de prueba (balance de comprobación) respetando el orden de las columnas, Esta información deberá estar por tres años y por meses, comenzando por el año actual y los dos años anteriores para las empresas y países que se vayan a consolidar</t>
-  </si>
-  <si>
-    <t>Z_Tipo</t>
-  </si>
-  <si>
-    <t>Z_Línea de negocio</t>
-  </si>
-  <si>
-    <t>Z_Ajuste1</t>
-  </si>
-  <si>
-    <t>Z_Ajuste2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Coloque el nombre de las líneas de venta que se hayan definido previamente. Estos nombres deberán ser siempre idénticos a la forma en que se reportarán en las bases de datos. </t>
-  </si>
-  <si>
-    <t>Coloque la clasificación de los costos y los gastos según su naturaleza así:</t>
   </si>
   <si>
     <t xml:space="preserve">En la columna C (Tipo) Coloque el nombre de las líneas de venta que se hayan definido previamente. Estos nombres deberán ser siempre idénticos a la forma en que se reportarán en las bases de datos. </t>
@@ -282,12 +201,6 @@
   </si>
   <si>
     <t>Así se usan cada una de las pestañas:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Coloque el nombre de las líneas de negocio que se hayan definido previamente. Estos nombres deberán ser siempre idénticos a la forma en que se reportarán en las bases de datos. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Coloque si el ingreso o el gasto se considera parte del Ebitda o no hace parte de él. Debe indicar siempre: </t>
   </si>
   <si>
     <r>
@@ -352,12 +265,6 @@
     <t>Las cuentas de Z_EjecPCH deben estar a de 4 a 6 dígitos del PUC y equivalen a los ahorros que ejecutados</t>
   </si>
   <si>
-    <t>Coloque la nomenclatura de la moneda en la cual se reportarán los datos eligiéndola de la lista desplegable</t>
-  </si>
-  <si>
-    <t>Elija de la lista desplegable</t>
-  </si>
-  <si>
     <t>En la columna K deberá indicar si el activo o el pasivo es corriente o no corriente para lo cual deberá usar la descripción de Z_Categorias USANDO LA LISTA DESPLEGABLE</t>
   </si>
   <si>
@@ -365,9 +272,6 @@
   </si>
   <si>
     <t>En la columna K Ajuste2 Coloque la clasificación de los costos y los gastos según su naturaleza así: USANDO LA LISTA DESPLEGABLE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Coloque el nombre de los países a consolidar. Estos nombres deberán ser siempre idénticos a la forma en que se reportarán en las bases de datos. Coloque el nombre con maýuscula solo en la primera letra y si tiene acento lo debes incluir. Ejem: Perú, México. </t>
   </si>
   <si>
     <t>Z_PresupuestoBalance</t>
@@ -721,7 +625,7 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -761,9 +665,6 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="183">
@@ -972,10 +873,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1339,7 +1236,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B746BB9-28D1-4089-9539-F175A9784447}">
-  <dimension ref="A1:X290"/>
+  <dimension ref="A1:X266"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="3.7109375" style="4" customWidth="1"/>
@@ -1380,7 +1277,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>51</v>
+        <v>24</v>
       </c>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
@@ -1408,7 +1305,7 @@
       <c r="A3" s="1"/>
       <c r="B3" s="2"/>
       <c r="C3" s="6" t="s">
-        <v>52</v>
+        <v>25</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -1436,7 +1333,7 @@
       <c r="A4" s="1"/>
       <c r="B4" s="7"/>
       <c r="C4" s="8" t="s">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
@@ -1490,7 +1387,7 @@
       <c r="A6" s="1"/>
       <c r="B6" s="2"/>
       <c r="C6" s="9" t="s">
-        <v>53</v>
+        <v>26</v>
       </c>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
@@ -1520,7 +1417,7 @@
         <v>1</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
@@ -1550,7 +1447,7 @@
         <v>2</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
@@ -1580,7 +1477,7 @@
         <v>3</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
@@ -1610,7 +1507,7 @@
         <v>4</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
@@ -1640,7 +1537,7 @@
         <v>5</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
@@ -1670,7 +1567,7 @@
         <v>6</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>54</v>
+        <v>27</v>
       </c>
       <c r="D12" s="1"/>
       <c r="E12" s="1"/>
@@ -1700,7 +1597,7 @@
         <v>7</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
@@ -1730,7 +1627,7 @@
         <v>8</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="D14" s="1"/>
       <c r="E14" s="1"/>
@@ -1760,7 +1657,7 @@
         <v>9</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>61</v>
+        <v>32</v>
       </c>
       <c r="D15" s="1"/>
       <c r="E15" s="1"/>
@@ -1790,7 +1687,7 @@
         <v>10</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>60</v>
+        <v>31</v>
       </c>
       <c r="D16" s="1"/>
       <c r="E16" s="1"/>
@@ -1844,7 +1741,7 @@
       <c r="A18" s="1"/>
       <c r="B18" s="10"/>
       <c r="C18" s="9" t="s">
-        <v>56</v>
+        <v>29</v>
       </c>
       <c r="D18" s="1"/>
       <c r="E18" s="1"/>
@@ -1871,10 +1768,10 @@
     <row r="19" spans="1:24" ht="15">
       <c r="A19" s="1"/>
       <c r="B19" s="11" t="s">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="D19" s="1"/>
       <c r="E19" s="1"/>
@@ -1900,11 +1797,9 @@
     </row>
     <row r="20" spans="1:24" ht="15">
       <c r="A20" s="1"/>
-      <c r="B20" s="11" t="s">
-        <v>17</v>
-      </c>
+      <c r="B20" s="11"/>
       <c r="C20" s="3" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="D20" s="1"/>
       <c r="E20" s="1"/>
@@ -1928,13 +1823,11 @@
       <c r="W20" s="1"/>
       <c r="X20" s="1"/>
     </row>
-    <row r="21" spans="1:24" ht="28.5">
+    <row r="21" spans="1:24" ht="15">
       <c r="A21" s="1"/>
-      <c r="B21" s="11" t="s">
-        <v>18</v>
-      </c>
+      <c r="B21" s="11"/>
       <c r="C21" s="3" t="s">
-        <v>80</v>
+        <v>15</v>
       </c>
       <c r="D21" s="1"/>
       <c r="E21" s="1"/>
@@ -1958,13 +1851,11 @@
       <c r="W21" s="1"/>
       <c r="X21" s="1"/>
     </row>
-    <row r="22" spans="1:24" ht="15">
+    <row r="22" spans="1:24" ht="28.5">
       <c r="A22" s="1"/>
-      <c r="B22" s="11" t="s">
+      <c r="B22" s="11"/>
+      <c r="C22" s="3" t="s">
         <v>19</v>
-      </c>
-      <c r="C22" s="3" t="s">
-        <v>30</v>
       </c>
       <c r="D22" s="1"/>
       <c r="E22" s="1"/>
@@ -1988,13 +1879,11 @@
       <c r="W22" s="1"/>
       <c r="X22" s="1"/>
     </row>
-    <row r="23" spans="1:24" ht="28.5">
+    <row r="23" spans="1:24" ht="15">
       <c r="A23" s="1"/>
-      <c r="B23" s="11" t="s">
-        <v>20</v>
-      </c>
+      <c r="B23" s="11"/>
       <c r="C23" s="3" t="s">
-        <v>31</v>
+        <v>53</v>
       </c>
       <c r="D23" s="1"/>
       <c r="E23" s="1"/>
@@ -2018,11 +1907,13 @@
       <c r="W23" s="1"/>
       <c r="X23" s="1"/>
     </row>
-    <row r="24" spans="1:24" ht="15">
+    <row r="24" spans="1:24" ht="28.5">
       <c r="A24" s="1"/>
-      <c r="B24" s="11"/>
+      <c r="B24" s="11" t="s">
+        <v>10</v>
+      </c>
       <c r="C24" s="3" t="s">
-        <v>5</v>
+        <v>56</v>
       </c>
       <c r="D24" s="1"/>
       <c r="E24" s="1"/>
@@ -2046,11 +1937,11 @@
       <c r="W24" s="1"/>
       <c r="X24" s="1"/>
     </row>
-    <row r="25" spans="1:24" ht="15">
+    <row r="25" spans="1:24" ht="28.5">
       <c r="A25" s="1"/>
       <c r="B25" s="11"/>
       <c r="C25" s="3" t="s">
-        <v>6</v>
+        <v>46</v>
       </c>
       <c r="D25" s="1"/>
       <c r="E25" s="1"/>
@@ -2078,7 +1969,7 @@
       <c r="A26" s="1"/>
       <c r="B26" s="11"/>
       <c r="C26" s="3" t="s">
-        <v>7</v>
+        <v>33</v>
       </c>
       <c r="D26" s="1"/>
       <c r="E26" s="1"/>
@@ -2104,9 +1995,11 @@
     </row>
     <row r="27" spans="1:24" ht="15">
       <c r="A27" s="1"/>
-      <c r="B27" s="11"/>
+      <c r="B27" s="11" t="s">
+        <v>11</v>
+      </c>
       <c r="C27" s="3" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="D27" s="1"/>
       <c r="E27" s="1"/>
@@ -2132,11 +2025,9 @@
     </row>
     <row r="28" spans="1:24" ht="15">
       <c r="A28" s="1"/>
-      <c r="B28" s="11" t="s">
-        <v>21</v>
-      </c>
+      <c r="B28" s="11"/>
       <c r="C28" s="3" t="s">
-        <v>75</v>
+        <v>18</v>
       </c>
       <c r="D28" s="1"/>
       <c r="E28" s="1"/>
@@ -2162,11 +2053,9 @@
     </row>
     <row r="29" spans="1:24" ht="15">
       <c r="A29" s="1"/>
-      <c r="B29" s="11" t="s">
-        <v>22</v>
-      </c>
+      <c r="B29" s="11"/>
       <c r="C29" s="3" t="s">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="D29" s="1"/>
       <c r="E29" s="1"/>
@@ -2194,7 +2083,7 @@
       <c r="A30" s="1"/>
       <c r="B30" s="11"/>
       <c r="C30" s="3" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="D30" s="1"/>
       <c r="E30" s="1"/>
@@ -2218,11 +2107,11 @@
       <c r="W30" s="1"/>
       <c r="X30" s="1"/>
     </row>
-    <row r="31" spans="1:24" ht="15">
+    <row r="31" spans="1:24" ht="28.5">
       <c r="A31" s="1"/>
       <c r="B31" s="11"/>
       <c r="C31" s="3" t="s">
-        <v>33</v>
+        <v>55</v>
       </c>
       <c r="D31" s="1"/>
       <c r="E31" s="1"/>
@@ -2246,11 +2135,11 @@
       <c r="W31" s="1"/>
       <c r="X31" s="1"/>
     </row>
-    <row r="32" spans="1:24" ht="15">
+    <row r="32" spans="1:24" ht="28.5">
       <c r="A32" s="1"/>
       <c r="B32" s="11"/>
       <c r="C32" s="3" t="s">
-        <v>34</v>
+        <v>20</v>
       </c>
       <c r="D32" s="1"/>
       <c r="E32" s="1"/>
@@ -2274,11 +2163,11 @@
       <c r="W32" s="1"/>
       <c r="X32" s="1"/>
     </row>
-    <row r="33" spans="1:24" ht="15">
+    <row r="33" spans="1:24" ht="28.5">
       <c r="A33" s="1"/>
       <c r="B33" s="11"/>
       <c r="C33" s="3" t="s">
-        <v>76</v>
+        <v>21</v>
       </c>
       <c r="D33" s="1"/>
       <c r="E33" s="1"/>
@@ -2304,11 +2193,9 @@
     </row>
     <row r="34" spans="1:24" ht="28.5">
       <c r="A34" s="1"/>
-      <c r="B34" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="C34" s="16" t="s">
-        <v>45</v>
+      <c r="B34" s="11"/>
+      <c r="C34" s="3" t="s">
+        <v>47</v>
       </c>
       <c r="D34" s="1"/>
       <c r="E34" s="1"/>
@@ -2332,13 +2219,11 @@
       <c r="W34" s="1"/>
       <c r="X34" s="1"/>
     </row>
-    <row r="35" spans="1:24" ht="28.5">
+    <row r="35" spans="1:24" ht="15">
       <c r="A35" s="1"/>
-      <c r="B35" s="11" t="s">
-        <v>42</v>
-      </c>
+      <c r="B35" s="11"/>
       <c r="C35" s="3" t="s">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="D35" s="1"/>
       <c r="E35" s="1"/>
@@ -2364,11 +2249,9 @@
     </row>
     <row r="36" spans="1:24" ht="15">
       <c r="A36" s="1"/>
-      <c r="B36" s="11" t="s">
-        <v>43</v>
-      </c>
+      <c r="B36" s="11"/>
       <c r="C36" s="3" t="s">
-        <v>58</v>
+        <v>0</v>
       </c>
       <c r="D36" s="1"/>
       <c r="E36" s="1"/>
@@ -2396,7 +2279,7 @@
       <c r="A37" s="1"/>
       <c r="B37" s="11"/>
       <c r="C37" s="3" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D37" s="1"/>
       <c r="E37" s="1"/>
@@ -2424,7 +2307,7 @@
       <c r="A38" s="1"/>
       <c r="B38" s="11"/>
       <c r="C38" s="3" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D38" s="1"/>
       <c r="E38" s="1"/>
@@ -2450,11 +2333,9 @@
     </row>
     <row r="39" spans="1:24" ht="15">
       <c r="A39" s="1"/>
-      <c r="B39" s="11" t="s">
-        <v>44</v>
-      </c>
+      <c r="B39" s="11"/>
       <c r="C39" s="3" t="s">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="D39" s="1"/>
       <c r="E39" s="1"/>
@@ -2480,9 +2361,11 @@
     </row>
     <row r="40" spans="1:24" ht="15">
       <c r="A40" s="1"/>
-      <c r="B40" s="11"/>
+      <c r="B40" s="11" t="s">
+        <v>12</v>
+      </c>
       <c r="C40" s="3" t="s">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="D40" s="1"/>
       <c r="E40" s="1"/>
@@ -2510,7 +2393,7 @@
       <c r="A41" s="1"/>
       <c r="B41" s="11"/>
       <c r="C41" s="3" t="s">
-        <v>1</v>
+        <v>36</v>
       </c>
       <c r="D41" s="1"/>
       <c r="E41" s="1"/>
@@ -2534,11 +2417,13 @@
       <c r="W41" s="1"/>
       <c r="X41" s="1"/>
     </row>
-    <row r="42" spans="1:24" ht="15">
+    <row r="42" spans="1:24" ht="28.5">
       <c r="A42" s="1"/>
-      <c r="B42" s="11"/>
+      <c r="B42" s="11" t="s">
+        <v>49</v>
+      </c>
       <c r="C42" s="3" t="s">
-        <v>2</v>
+        <v>54</v>
       </c>
       <c r="D42" s="1"/>
       <c r="E42" s="1"/>
@@ -2564,11 +2449,9 @@
     </row>
     <row r="43" spans="1:24" ht="15">
       <c r="A43" s="1"/>
-      <c r="B43" s="11" t="s">
-        <v>23</v>
-      </c>
+      <c r="B43" s="11"/>
       <c r="C43" s="3" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D43" s="1"/>
       <c r="E43" s="1"/>
@@ -2594,9 +2477,11 @@
     </row>
     <row r="44" spans="1:24" ht="15">
       <c r="A44" s="1"/>
-      <c r="B44" s="11"/>
+      <c r="B44" s="11" t="s">
+        <v>51</v>
+      </c>
       <c r="C44" s="3" t="s">
-        <v>35</v>
+        <v>22</v>
       </c>
       <c r="D44" s="1"/>
       <c r="E44" s="1"/>
@@ -2624,7 +2509,7 @@
       <c r="A45" s="1"/>
       <c r="B45" s="11"/>
       <c r="C45" s="3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D45" s="1"/>
       <c r="E45" s="1"/>
@@ -2648,11 +2533,13 @@
       <c r="W45" s="1"/>
       <c r="X45" s="1"/>
     </row>
-    <row r="46" spans="1:24" ht="28.5">
+    <row r="46" spans="1:24" ht="15">
       <c r="A46" s="1"/>
-      <c r="B46" s="11"/>
+      <c r="B46" s="11" t="s">
+        <v>52</v>
+      </c>
       <c r="C46" s="3" t="s">
-        <v>40</v>
+        <v>23</v>
       </c>
       <c r="D46" s="1"/>
       <c r="E46" s="1"/>
@@ -2680,7 +2567,7 @@
       <c r="A47" s="1"/>
       <c r="B47" s="11"/>
       <c r="C47" s="3" t="s">
-        <v>85</v>
+        <v>38</v>
       </c>
       <c r="D47" s="1"/>
       <c r="E47" s="1"/>
@@ -2704,13 +2591,13 @@
       <c r="W47" s="1"/>
       <c r="X47" s="1"/>
     </row>
-    <row r="48" spans="1:24" ht="28.5">
+    <row r="48" spans="1:24" ht="15">
       <c r="A48" s="1"/>
       <c r="B48" s="11" t="s">
-        <v>24</v>
+        <v>40</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>88</v>
+        <v>43</v>
       </c>
       <c r="D48" s="1"/>
       <c r="E48" s="1"/>
@@ -2734,11 +2621,11 @@
       <c r="W48" s="1"/>
       <c r="X48" s="1"/>
     </row>
-    <row r="49" spans="1:24" ht="28.5">
+    <row r="49" spans="1:24" ht="15">
       <c r="A49" s="1"/>
       <c r="B49" s="11"/>
       <c r="C49" s="3" t="s">
-        <v>77</v>
+        <v>42</v>
       </c>
       <c r="D49" s="1"/>
       <c r="E49" s="1"/>
@@ -2764,9 +2651,11 @@
     </row>
     <row r="50" spans="1:24" ht="15">
       <c r="A50" s="1"/>
-      <c r="B50" s="11"/>
+      <c r="B50" s="11" t="s">
+        <v>41</v>
+      </c>
       <c r="C50" s="3" t="s">
-        <v>62</v>
+        <v>44</v>
       </c>
       <c r="D50" s="1"/>
       <c r="E50" s="1"/>
@@ -2792,11 +2681,9 @@
     </row>
     <row r="51" spans="1:24" ht="15">
       <c r="A51" s="1"/>
-      <c r="B51" s="11" t="s">
-        <v>25</v>
-      </c>
+      <c r="B51" s="11"/>
       <c r="C51" s="3" t="s">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="D51" s="1"/>
       <c r="E51" s="1"/>
@@ -2822,7 +2709,9 @@
     </row>
     <row r="52" spans="1:24" ht="15">
       <c r="A52" s="1"/>
-      <c r="B52" s="11"/>
+      <c r="B52" s="11" t="s">
+        <v>13</v>
+      </c>
       <c r="C52" s="3" t="s">
         <v>39</v>
       </c>
@@ -2848,12 +2737,10 @@
       <c r="W52" s="1"/>
       <c r="X52" s="1"/>
     </row>
-    <row r="53" spans="1:24" ht="15">
+    <row r="53" spans="1:24">
       <c r="A53" s="1"/>
-      <c r="B53" s="11"/>
-      <c r="C53" s="3" t="s">
-        <v>35</v>
-      </c>
+      <c r="B53" s="2"/>
+      <c r="C53" s="3"/>
       <c r="D53" s="1"/>
       <c r="E53" s="1"/>
       <c r="F53" s="1"/>
@@ -2876,12 +2763,8 @@
       <c r="W53" s="1"/>
       <c r="X53" s="1"/>
     </row>
-    <row r="54" spans="1:24" ht="15">
+    <row r="54" spans="1:24">
       <c r="A54" s="1"/>
-      <c r="B54" s="11"/>
-      <c r="C54" s="3" t="s">
-        <v>36</v>
-      </c>
       <c r="D54" s="1"/>
       <c r="E54" s="1"/>
       <c r="F54" s="1"/>
@@ -2904,12 +2787,8 @@
       <c r="W54" s="1"/>
       <c r="X54" s="1"/>
     </row>
-    <row r="55" spans="1:24" ht="28.5">
+    <row r="55" spans="1:24">
       <c r="A55" s="1"/>
-      <c r="B55" s="11"/>
-      <c r="C55" s="3" t="s">
-        <v>87</v>
-      </c>
       <c r="D55" s="1"/>
       <c r="E55" s="1"/>
       <c r="F55" s="1"/>
@@ -2932,12 +2811,8 @@
       <c r="W55" s="1"/>
       <c r="X55" s="1"/>
     </row>
-    <row r="56" spans="1:24" ht="28.5">
+    <row r="56" spans="1:24">
       <c r="A56" s="1"/>
-      <c r="B56" s="11"/>
-      <c r="C56" s="3" t="s">
-        <v>47</v>
-      </c>
       <c r="D56" s="1"/>
       <c r="E56" s="1"/>
       <c r="F56" s="1"/>
@@ -2960,12 +2835,8 @@
       <c r="W56" s="1"/>
       <c r="X56" s="1"/>
     </row>
-    <row r="57" spans="1:24" ht="28.5">
+    <row r="57" spans="1:24">
       <c r="A57" s="1"/>
-      <c r="B57" s="11"/>
-      <c r="C57" s="3" t="s">
-        <v>48</v>
-      </c>
       <c r="D57" s="1"/>
       <c r="E57" s="1"/>
       <c r="F57" s="1"/>
@@ -2988,12 +2859,8 @@
       <c r="W57" s="1"/>
       <c r="X57" s="1"/>
     </row>
-    <row r="58" spans="1:24" ht="28.5">
+    <row r="58" spans="1:24">
       <c r="A58" s="1"/>
-      <c r="B58" s="11"/>
-      <c r="C58" s="3" t="s">
-        <v>78</v>
-      </c>
       <c r="D58" s="1"/>
       <c r="E58" s="1"/>
       <c r="F58" s="1"/>
@@ -3016,679 +2883,603 @@
       <c r="W58" s="1"/>
       <c r="X58" s="1"/>
     </row>
-    <row r="59" spans="1:24" ht="15">
-      <c r="A59" s="1"/>
-      <c r="B59" s="11"/>
-      <c r="C59" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="D59" s="1"/>
-      <c r="E59" s="1"/>
-      <c r="F59" s="1"/>
-      <c r="G59" s="1"/>
-      <c r="H59" s="1"/>
-      <c r="I59" s="1"/>
-      <c r="J59" s="1"/>
-      <c r="K59" s="1"/>
-      <c r="L59" s="1"/>
-      <c r="M59" s="1"/>
-      <c r="N59" s="1"/>
-      <c r="O59" s="1"/>
-      <c r="P59" s="1"/>
-      <c r="Q59" s="1"/>
-      <c r="R59" s="1"/>
-      <c r="S59" s="1"/>
-      <c r="T59" s="1"/>
-      <c r="U59" s="1"/>
-      <c r="V59" s="1"/>
-      <c r="W59" s="1"/>
-      <c r="X59" s="1"/>
-    </row>
-    <row r="60" spans="1:24" ht="15">
-      <c r="A60" s="1"/>
-      <c r="B60" s="11"/>
-      <c r="C60" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="D60" s="1"/>
-      <c r="E60" s="1"/>
-      <c r="F60" s="1"/>
-      <c r="G60" s="1"/>
-      <c r="H60" s="1"/>
-      <c r="I60" s="1"/>
-      <c r="J60" s="1"/>
-      <c r="K60" s="1"/>
-      <c r="L60" s="1"/>
-      <c r="M60" s="1"/>
-      <c r="N60" s="1"/>
-      <c r="O60" s="1"/>
-      <c r="P60" s="1"/>
-      <c r="Q60" s="1"/>
-      <c r="R60" s="1"/>
-      <c r="S60" s="1"/>
-      <c r="T60" s="1"/>
-      <c r="U60" s="1"/>
-      <c r="V60" s="1"/>
-      <c r="W60" s="1"/>
-      <c r="X60" s="1"/>
-    </row>
-    <row r="61" spans="1:24" ht="15">
-      <c r="A61" s="1"/>
-      <c r="B61" s="11"/>
-      <c r="C61" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="D61" s="1"/>
-      <c r="E61" s="1"/>
-      <c r="F61" s="1"/>
-      <c r="G61" s="1"/>
-      <c r="H61" s="1"/>
-      <c r="I61" s="1"/>
-      <c r="J61" s="1"/>
-      <c r="K61" s="1"/>
-      <c r="L61" s="1"/>
-      <c r="M61" s="1"/>
-      <c r="N61" s="1"/>
-      <c r="O61" s="1"/>
-      <c r="P61" s="1"/>
-      <c r="Q61" s="1"/>
-      <c r="R61" s="1"/>
-      <c r="S61" s="1"/>
-      <c r="T61" s="1"/>
-      <c r="U61" s="1"/>
-      <c r="V61" s="1"/>
-      <c r="W61" s="1"/>
-      <c r="X61" s="1"/>
-    </row>
-    <row r="62" spans="1:24" ht="15">
-      <c r="A62" s="1"/>
-      <c r="B62" s="11"/>
-      <c r="C62" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="D62" s="1"/>
-      <c r="E62" s="1"/>
-      <c r="F62" s="1"/>
-      <c r="G62" s="1"/>
-      <c r="H62" s="1"/>
-      <c r="I62" s="1"/>
-      <c r="J62" s="1"/>
-      <c r="K62" s="1"/>
-      <c r="L62" s="1"/>
-      <c r="M62" s="1"/>
-      <c r="N62" s="1"/>
-      <c r="O62" s="1"/>
-      <c r="P62" s="1"/>
-      <c r="Q62" s="1"/>
-      <c r="R62" s="1"/>
-      <c r="S62" s="1"/>
-      <c r="T62" s="1"/>
-      <c r="U62" s="1"/>
-      <c r="V62" s="1"/>
-      <c r="W62" s="1"/>
-      <c r="X62" s="1"/>
-    </row>
-    <row r="63" spans="1:24" ht="15">
-      <c r="A63" s="1"/>
-      <c r="B63" s="11"/>
-      <c r="C63" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="D63" s="1"/>
-      <c r="E63" s="1"/>
-      <c r="F63" s="1"/>
-      <c r="G63" s="1"/>
-      <c r="H63" s="1"/>
-      <c r="I63" s="1"/>
-      <c r="J63" s="1"/>
-      <c r="K63" s="1"/>
-      <c r="L63" s="1"/>
-      <c r="M63" s="1"/>
-      <c r="N63" s="1"/>
-      <c r="O63" s="1"/>
-      <c r="P63" s="1"/>
-      <c r="Q63" s="1"/>
-      <c r="R63" s="1"/>
-      <c r="S63" s="1"/>
-      <c r="T63" s="1"/>
-      <c r="U63" s="1"/>
-      <c r="V63" s="1"/>
-      <c r="W63" s="1"/>
-      <c r="X63" s="1"/>
-    </row>
-    <row r="64" spans="1:24" ht="15">
-      <c r="A64" s="1"/>
-      <c r="B64" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="C64" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="D64" s="1"/>
-      <c r="E64" s="1"/>
-      <c r="F64" s="1"/>
-      <c r="G64" s="1"/>
-      <c r="H64" s="1"/>
-      <c r="I64" s="1"/>
-      <c r="J64" s="1"/>
-      <c r="K64" s="1"/>
-      <c r="L64" s="1"/>
-      <c r="M64" s="1"/>
-      <c r="N64" s="1"/>
-      <c r="O64" s="1"/>
-      <c r="P64" s="1"/>
-      <c r="Q64" s="1"/>
-      <c r="R64" s="1"/>
-      <c r="S64" s="1"/>
-      <c r="T64" s="1"/>
-      <c r="U64" s="1"/>
-      <c r="V64" s="1"/>
-      <c r="W64" s="1"/>
-      <c r="X64" s="1"/>
-    </row>
-    <row r="65" spans="1:24" ht="15">
-      <c r="A65" s="1"/>
-      <c r="B65" s="11"/>
-      <c r="C65" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="D65" s="1"/>
-      <c r="E65" s="1"/>
-      <c r="F65" s="1"/>
-      <c r="G65" s="1"/>
-      <c r="H65" s="1"/>
-      <c r="I65" s="1"/>
-      <c r="J65" s="1"/>
-      <c r="K65" s="1"/>
-      <c r="L65" s="1"/>
-      <c r="M65" s="1"/>
-      <c r="N65" s="1"/>
-      <c r="O65" s="1"/>
-      <c r="P65" s="1"/>
-      <c r="Q65" s="1"/>
-      <c r="R65" s="1"/>
-      <c r="S65" s="1"/>
-      <c r="T65" s="1"/>
-      <c r="U65" s="1"/>
-      <c r="V65" s="1"/>
-      <c r="W65" s="1"/>
-      <c r="X65" s="1"/>
-    </row>
-    <row r="66" spans="1:24" ht="28.5">
-      <c r="A66" s="1"/>
-      <c r="B66" s="11" t="s">
-        <v>81</v>
-      </c>
-      <c r="C66" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="D66" s="1"/>
-      <c r="E66" s="1"/>
-      <c r="F66" s="1"/>
-      <c r="G66" s="1"/>
-      <c r="H66" s="1"/>
-      <c r="I66" s="1"/>
-      <c r="J66" s="1"/>
-      <c r="K66" s="1"/>
-      <c r="L66" s="1"/>
-      <c r="M66" s="1"/>
-      <c r="N66" s="1"/>
-      <c r="O66" s="1"/>
-      <c r="P66" s="1"/>
-      <c r="Q66" s="1"/>
-      <c r="R66" s="1"/>
-      <c r="S66" s="1"/>
-      <c r="T66" s="1"/>
-      <c r="U66" s="1"/>
-      <c r="V66" s="1"/>
-      <c r="W66" s="1"/>
-      <c r="X66" s="1"/>
-    </row>
-    <row r="67" spans="1:24" ht="15">
-      <c r="A67" s="1"/>
-      <c r="B67" s="11"/>
-      <c r="C67" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="D67" s="1"/>
-      <c r="E67" s="1"/>
-      <c r="F67" s="1"/>
-      <c r="G67" s="1"/>
-      <c r="H67" s="1"/>
-      <c r="I67" s="1"/>
-      <c r="J67" s="1"/>
-      <c r="K67" s="1"/>
-      <c r="L67" s="1"/>
-      <c r="M67" s="1"/>
-      <c r="N67" s="1"/>
-      <c r="O67" s="1"/>
-      <c r="P67" s="1"/>
-      <c r="Q67" s="1"/>
-      <c r="R67" s="1"/>
-      <c r="S67" s="1"/>
-      <c r="T67" s="1"/>
-      <c r="U67" s="1"/>
-      <c r="V67" s="1"/>
-      <c r="W67" s="1"/>
-      <c r="X67" s="1"/>
-    </row>
-    <row r="68" spans="1:24" ht="15">
-      <c r="A68" s="1"/>
-      <c r="B68" s="11" t="s">
-        <v>83</v>
-      </c>
-      <c r="C68" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="D68" s="1"/>
-      <c r="E68" s="1"/>
-      <c r="F68" s="1"/>
-      <c r="G68" s="1"/>
-      <c r="H68" s="1"/>
-      <c r="I68" s="1"/>
-      <c r="J68" s="1"/>
-      <c r="K68" s="1"/>
-      <c r="L68" s="1"/>
-      <c r="M68" s="1"/>
-      <c r="N68" s="1"/>
-      <c r="O68" s="1"/>
-      <c r="P68" s="1"/>
-      <c r="Q68" s="1"/>
-      <c r="R68" s="1"/>
-      <c r="S68" s="1"/>
-      <c r="T68" s="1"/>
-      <c r="U68" s="1"/>
-      <c r="V68" s="1"/>
-      <c r="W68" s="1"/>
-      <c r="X68" s="1"/>
-    </row>
-    <row r="69" spans="1:24" ht="15">
-      <c r="A69" s="1"/>
-      <c r="B69" s="11"/>
-      <c r="C69" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="D69" s="1"/>
-      <c r="E69" s="1"/>
-      <c r="F69" s="1"/>
-      <c r="G69" s="1"/>
-      <c r="H69" s="1"/>
-      <c r="I69" s="1"/>
-      <c r="J69" s="1"/>
-      <c r="K69" s="1"/>
-      <c r="L69" s="1"/>
-      <c r="M69" s="1"/>
-      <c r="N69" s="1"/>
-      <c r="O69" s="1"/>
-      <c r="P69" s="1"/>
-      <c r="Q69" s="1"/>
-      <c r="R69" s="1"/>
-      <c r="S69" s="1"/>
-      <c r="T69" s="1"/>
-      <c r="U69" s="1"/>
-      <c r="V69" s="1"/>
-      <c r="W69" s="1"/>
-      <c r="X69" s="1"/>
-    </row>
-    <row r="70" spans="1:24" ht="15">
-      <c r="A70" s="1"/>
-      <c r="B70" s="11" t="s">
-        <v>84</v>
-      </c>
-      <c r="C70" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="D70" s="1"/>
-      <c r="E70" s="1"/>
-      <c r="F70" s="1"/>
-      <c r="G70" s="1"/>
-      <c r="H70" s="1"/>
-      <c r="I70" s="1"/>
-      <c r="J70" s="1"/>
-      <c r="K70" s="1"/>
-      <c r="L70" s="1"/>
-      <c r="M70" s="1"/>
-      <c r="N70" s="1"/>
-      <c r="O70" s="1"/>
-      <c r="P70" s="1"/>
-      <c r="Q70" s="1"/>
-      <c r="R70" s="1"/>
-      <c r="S70" s="1"/>
-      <c r="T70" s="1"/>
-      <c r="U70" s="1"/>
-      <c r="V70" s="1"/>
-      <c r="W70" s="1"/>
-      <c r="X70" s="1"/>
-    </row>
-    <row r="71" spans="1:24" ht="15">
-      <c r="A71" s="1"/>
-      <c r="B71" s="11"/>
-      <c r="C71" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="D71" s="1"/>
-      <c r="E71" s="1"/>
-      <c r="F71" s="1"/>
-      <c r="G71" s="1"/>
-      <c r="H71" s="1"/>
-      <c r="I71" s="1"/>
-      <c r="J71" s="1"/>
-      <c r="K71" s="1"/>
-      <c r="L71" s="1"/>
-      <c r="M71" s="1"/>
-      <c r="N71" s="1"/>
-      <c r="O71" s="1"/>
-      <c r="P71" s="1"/>
-      <c r="Q71" s="1"/>
-      <c r="R71" s="1"/>
-      <c r="S71" s="1"/>
-      <c r="T71" s="1"/>
-      <c r="U71" s="1"/>
-      <c r="V71" s="1"/>
-      <c r="W71" s="1"/>
-      <c r="X71" s="1"/>
-    </row>
-    <row r="72" spans="1:24" ht="15">
-      <c r="A72" s="1"/>
-      <c r="B72" s="11" t="s">
-        <v>69</v>
-      </c>
-      <c r="C72" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="D72" s="1"/>
-      <c r="E72" s="1"/>
-      <c r="F72" s="1"/>
-      <c r="G72" s="1"/>
-      <c r="H72" s="1"/>
-      <c r="I72" s="1"/>
-      <c r="J72" s="1"/>
-      <c r="K72" s="1"/>
-      <c r="L72" s="1"/>
-      <c r="M72" s="1"/>
-      <c r="N72" s="1"/>
-      <c r="O72" s="1"/>
-      <c r="P72" s="1"/>
-      <c r="Q72" s="1"/>
-      <c r="R72" s="1"/>
-      <c r="S72" s="1"/>
-      <c r="T72" s="1"/>
-      <c r="U72" s="1"/>
-      <c r="V72" s="1"/>
-      <c r="W72" s="1"/>
-      <c r="X72" s="1"/>
-    </row>
-    <row r="73" spans="1:24" ht="15">
-      <c r="A73" s="1"/>
-      <c r="B73" s="11"/>
-      <c r="C73" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="D73" s="1"/>
-      <c r="E73" s="1"/>
-      <c r="F73" s="1"/>
-      <c r="G73" s="1"/>
-      <c r="H73" s="1"/>
-      <c r="I73" s="1"/>
-      <c r="J73" s="1"/>
-      <c r="K73" s="1"/>
-      <c r="L73" s="1"/>
-      <c r="M73" s="1"/>
-      <c r="N73" s="1"/>
-      <c r="O73" s="1"/>
-      <c r="P73" s="1"/>
-      <c r="Q73" s="1"/>
-      <c r="R73" s="1"/>
-      <c r="S73" s="1"/>
-      <c r="T73" s="1"/>
-      <c r="U73" s="1"/>
-      <c r="V73" s="1"/>
-      <c r="W73" s="1"/>
-      <c r="X73" s="1"/>
-    </row>
-    <row r="74" spans="1:24" ht="15">
-      <c r="A74" s="1"/>
-      <c r="B74" s="11" t="s">
-        <v>70</v>
-      </c>
-      <c r="C74" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="D74" s="1"/>
-      <c r="E74" s="1"/>
-      <c r="F74" s="1"/>
-      <c r="G74" s="1"/>
-      <c r="H74" s="1"/>
-      <c r="I74" s="1"/>
-      <c r="J74" s="1"/>
-      <c r="K74" s="1"/>
-      <c r="L74" s="1"/>
-      <c r="M74" s="1"/>
-      <c r="N74" s="1"/>
-      <c r="O74" s="1"/>
-      <c r="P74" s="1"/>
-      <c r="Q74" s="1"/>
-      <c r="R74" s="1"/>
-      <c r="S74" s="1"/>
-      <c r="T74" s="1"/>
-      <c r="U74" s="1"/>
-      <c r="V74" s="1"/>
-      <c r="W74" s="1"/>
-      <c r="X74" s="1"/>
-    </row>
-    <row r="75" spans="1:24" ht="15">
-      <c r="A75" s="1"/>
-      <c r="B75" s="11"/>
-      <c r="C75" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="D75" s="1"/>
-      <c r="E75" s="1"/>
-      <c r="F75" s="1"/>
-      <c r="G75" s="1"/>
-      <c r="H75" s="1"/>
-      <c r="I75" s="1"/>
-      <c r="J75" s="1"/>
-      <c r="K75" s="1"/>
-      <c r="L75" s="1"/>
-      <c r="M75" s="1"/>
-      <c r="N75" s="1"/>
-      <c r="O75" s="1"/>
-      <c r="P75" s="1"/>
-      <c r="Q75" s="1"/>
-      <c r="R75" s="1"/>
-      <c r="S75" s="1"/>
-      <c r="T75" s="1"/>
-      <c r="U75" s="1"/>
-      <c r="V75" s="1"/>
-      <c r="W75" s="1"/>
-      <c r="X75" s="1"/>
-    </row>
-    <row r="76" spans="1:24" ht="15">
-      <c r="A76" s="1"/>
-      <c r="B76" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="C76" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="D76" s="1"/>
-      <c r="E76" s="1"/>
-      <c r="F76" s="1"/>
-      <c r="G76" s="1"/>
-      <c r="H76" s="1"/>
-      <c r="I76" s="1"/>
-      <c r="J76" s="1"/>
-      <c r="K76" s="1"/>
-      <c r="L76" s="1"/>
-      <c r="M76" s="1"/>
-      <c r="N76" s="1"/>
-      <c r="O76" s="1"/>
-      <c r="P76" s="1"/>
-      <c r="Q76" s="1"/>
-      <c r="R76" s="1"/>
-      <c r="S76" s="1"/>
-      <c r="T76" s="1"/>
-      <c r="U76" s="1"/>
-      <c r="V76" s="1"/>
-      <c r="W76" s="1"/>
-      <c r="X76" s="1"/>
+    <row r="59" spans="1:24">
+      <c r="A59" s="12"/>
+      <c r="D59" s="12"/>
+      <c r="E59" s="12"/>
+      <c r="F59" s="12"/>
+      <c r="G59" s="12"/>
+      <c r="H59" s="12"/>
+      <c r="I59" s="12"/>
+      <c r="J59" s="12"/>
+      <c r="K59" s="12"/>
+      <c r="L59" s="12"/>
+      <c r="M59" s="12"/>
+      <c r="N59" s="12"/>
+      <c r="O59" s="12"/>
+      <c r="P59" s="12"/>
+      <c r="Q59" s="12"/>
+      <c r="R59" s="12"/>
+      <c r="S59" s="12"/>
+      <c r="T59" s="12"/>
+      <c r="U59" s="12"/>
+      <c r="V59" s="12"/>
+      <c r="W59" s="12"/>
+      <c r="X59" s="12"/>
+    </row>
+    <row r="60" spans="1:24">
+      <c r="A60" s="12"/>
+      <c r="D60" s="12"/>
+      <c r="E60" s="12"/>
+      <c r="F60" s="12"/>
+      <c r="G60" s="12"/>
+      <c r="H60" s="12"/>
+      <c r="I60" s="12"/>
+      <c r="J60" s="12"/>
+      <c r="K60" s="12"/>
+      <c r="L60" s="12"/>
+      <c r="M60" s="12"/>
+      <c r="N60" s="12"/>
+      <c r="O60" s="12"/>
+      <c r="P60" s="12"/>
+      <c r="Q60" s="12"/>
+      <c r="R60" s="12"/>
+      <c r="S60" s="12"/>
+      <c r="T60" s="12"/>
+      <c r="U60" s="12"/>
+      <c r="V60" s="12"/>
+      <c r="W60" s="12"/>
+      <c r="X60" s="12"/>
+    </row>
+    <row r="61" spans="1:24">
+      <c r="A61" s="12"/>
+      <c r="D61" s="12"/>
+      <c r="E61" s="12"/>
+      <c r="F61" s="12"/>
+      <c r="G61" s="12"/>
+      <c r="H61" s="12"/>
+      <c r="I61" s="12"/>
+      <c r="J61" s="12"/>
+      <c r="K61" s="12"/>
+      <c r="L61" s="12"/>
+      <c r="M61" s="12"/>
+      <c r="N61" s="12"/>
+      <c r="O61" s="12"/>
+      <c r="P61" s="12"/>
+      <c r="Q61" s="12"/>
+      <c r="R61" s="12"/>
+      <c r="S61" s="12"/>
+      <c r="T61" s="12"/>
+      <c r="U61" s="12"/>
+      <c r="V61" s="12"/>
+      <c r="W61" s="12"/>
+      <c r="X61" s="12"/>
+    </row>
+    <row r="62" spans="1:24">
+      <c r="A62" s="12"/>
+      <c r="D62" s="12"/>
+      <c r="E62" s="12"/>
+      <c r="F62" s="12"/>
+      <c r="G62" s="12"/>
+      <c r="H62" s="12"/>
+      <c r="I62" s="12"/>
+      <c r="J62" s="12"/>
+      <c r="K62" s="12"/>
+      <c r="L62" s="12"/>
+      <c r="M62" s="12"/>
+      <c r="N62" s="12"/>
+      <c r="O62" s="12"/>
+      <c r="P62" s="12"/>
+      <c r="Q62" s="12"/>
+      <c r="R62" s="12"/>
+      <c r="S62" s="12"/>
+      <c r="T62" s="12"/>
+      <c r="U62" s="12"/>
+      <c r="V62" s="12"/>
+      <c r="W62" s="12"/>
+      <c r="X62" s="12"/>
+    </row>
+    <row r="63" spans="1:24">
+      <c r="A63" s="12"/>
+      <c r="D63" s="12"/>
+      <c r="E63" s="12"/>
+      <c r="F63" s="12"/>
+      <c r="G63" s="12"/>
+      <c r="H63" s="12"/>
+      <c r="I63" s="12"/>
+      <c r="J63" s="12"/>
+      <c r="K63" s="12"/>
+      <c r="L63" s="12"/>
+      <c r="M63" s="12"/>
+      <c r="N63" s="12"/>
+      <c r="O63" s="12"/>
+      <c r="P63" s="12"/>
+      <c r="Q63" s="12"/>
+      <c r="R63" s="12"/>
+      <c r="S63" s="12"/>
+      <c r="T63" s="12"/>
+      <c r="U63" s="12"/>
+      <c r="V63" s="12"/>
+      <c r="W63" s="12"/>
+      <c r="X63" s="12"/>
+    </row>
+    <row r="64" spans="1:24">
+      <c r="A64" s="12"/>
+      <c r="D64" s="12"/>
+      <c r="E64" s="12"/>
+      <c r="F64" s="12"/>
+      <c r="G64" s="12"/>
+      <c r="H64" s="12"/>
+      <c r="I64" s="12"/>
+      <c r="J64" s="12"/>
+      <c r="K64" s="12"/>
+      <c r="L64" s="12"/>
+      <c r="M64" s="12"/>
+      <c r="N64" s="12"/>
+      <c r="O64" s="12"/>
+      <c r="P64" s="12"/>
+      <c r="Q64" s="12"/>
+      <c r="R64" s="12"/>
+      <c r="S64" s="12"/>
+      <c r="T64" s="12"/>
+      <c r="U64" s="12"/>
+      <c r="V64" s="12"/>
+      <c r="W64" s="12"/>
+      <c r="X64" s="12"/>
+    </row>
+    <row r="65" spans="1:24">
+      <c r="A65" s="12"/>
+      <c r="D65" s="12"/>
+      <c r="E65" s="12"/>
+      <c r="F65" s="12"/>
+      <c r="G65" s="12"/>
+      <c r="H65" s="12"/>
+      <c r="I65" s="12"/>
+      <c r="J65" s="12"/>
+      <c r="K65" s="12"/>
+      <c r="L65" s="12"/>
+      <c r="M65" s="12"/>
+      <c r="N65" s="12"/>
+      <c r="O65" s="12"/>
+      <c r="P65" s="12"/>
+      <c r="Q65" s="12"/>
+      <c r="R65" s="12"/>
+      <c r="S65" s="12"/>
+      <c r="T65" s="12"/>
+      <c r="U65" s="12"/>
+      <c r="V65" s="12"/>
+      <c r="W65" s="12"/>
+      <c r="X65" s="12"/>
+    </row>
+    <row r="66" spans="1:24">
+      <c r="A66" s="12"/>
+      <c r="D66" s="12"/>
+      <c r="E66" s="12"/>
+      <c r="F66" s="12"/>
+      <c r="G66" s="12"/>
+      <c r="H66" s="12"/>
+      <c r="I66" s="12"/>
+      <c r="J66" s="12"/>
+      <c r="K66" s="12"/>
+      <c r="L66" s="12"/>
+      <c r="M66" s="12"/>
+      <c r="N66" s="12"/>
+      <c r="O66" s="12"/>
+      <c r="P66" s="12"/>
+      <c r="Q66" s="12"/>
+      <c r="R66" s="12"/>
+      <c r="S66" s="12"/>
+      <c r="T66" s="12"/>
+      <c r="U66" s="12"/>
+      <c r="V66" s="12"/>
+      <c r="W66" s="12"/>
+      <c r="X66" s="12"/>
+    </row>
+    <row r="67" spans="1:24">
+      <c r="A67" s="12"/>
+      <c r="D67" s="12"/>
+      <c r="E67" s="12"/>
+      <c r="F67" s="12"/>
+      <c r="G67" s="12"/>
+      <c r="H67" s="12"/>
+      <c r="I67" s="12"/>
+      <c r="J67" s="12"/>
+      <c r="K67" s="12"/>
+      <c r="L67" s="12"/>
+      <c r="M67" s="12"/>
+      <c r="N67" s="12"/>
+      <c r="O67" s="12"/>
+      <c r="P67" s="12"/>
+      <c r="Q67" s="12"/>
+      <c r="R67" s="12"/>
+      <c r="S67" s="12"/>
+      <c r="T67" s="12"/>
+      <c r="U67" s="12"/>
+      <c r="V67" s="12"/>
+      <c r="W67" s="12"/>
+      <c r="X67" s="12"/>
+    </row>
+    <row r="68" spans="1:24">
+      <c r="A68" s="12"/>
+      <c r="D68" s="12"/>
+      <c r="E68" s="12"/>
+      <c r="F68" s="12"/>
+      <c r="G68" s="12"/>
+      <c r="H68" s="12"/>
+      <c r="I68" s="12"/>
+      <c r="J68" s="12"/>
+      <c r="K68" s="12"/>
+      <c r="L68" s="12"/>
+      <c r="M68" s="12"/>
+      <c r="N68" s="12"/>
+      <c r="O68" s="12"/>
+      <c r="P68" s="12"/>
+      <c r="Q68" s="12"/>
+      <c r="R68" s="12"/>
+      <c r="S68" s="12"/>
+      <c r="T68" s="12"/>
+      <c r="U68" s="12"/>
+      <c r="V68" s="12"/>
+      <c r="W68" s="12"/>
+      <c r="X68" s="12"/>
+    </row>
+    <row r="69" spans="1:24">
+      <c r="A69" s="12"/>
+      <c r="D69" s="12"/>
+      <c r="E69" s="12"/>
+      <c r="F69" s="12"/>
+      <c r="G69" s="12"/>
+      <c r="H69" s="12"/>
+      <c r="I69" s="12"/>
+      <c r="J69" s="12"/>
+      <c r="K69" s="12"/>
+      <c r="L69" s="12"/>
+      <c r="M69" s="12"/>
+      <c r="N69" s="12"/>
+      <c r="O69" s="12"/>
+      <c r="P69" s="12"/>
+      <c r="Q69" s="12"/>
+      <c r="R69" s="12"/>
+      <c r="S69" s="12"/>
+      <c r="T69" s="12"/>
+      <c r="U69" s="12"/>
+      <c r="V69" s="12"/>
+      <c r="W69" s="12"/>
+      <c r="X69" s="12"/>
+    </row>
+    <row r="70" spans="1:24">
+      <c r="A70" s="12"/>
+      <c r="D70" s="12"/>
+      <c r="E70" s="12"/>
+      <c r="F70" s="12"/>
+      <c r="G70" s="12"/>
+      <c r="H70" s="12"/>
+      <c r="I70" s="12"/>
+      <c r="J70" s="12"/>
+      <c r="K70" s="12"/>
+      <c r="L70" s="12"/>
+      <c r="M70" s="12"/>
+      <c r="N70" s="12"/>
+      <c r="O70" s="12"/>
+      <c r="P70" s="12"/>
+      <c r="Q70" s="12"/>
+      <c r="R70" s="12"/>
+      <c r="S70" s="12"/>
+      <c r="T70" s="12"/>
+      <c r="U70" s="12"/>
+      <c r="V70" s="12"/>
+      <c r="W70" s="12"/>
+      <c r="X70" s="12"/>
+    </row>
+    <row r="71" spans="1:24">
+      <c r="A71" s="12"/>
+      <c r="D71" s="12"/>
+      <c r="E71" s="12"/>
+      <c r="F71" s="12"/>
+      <c r="G71" s="12"/>
+      <c r="H71" s="12"/>
+      <c r="I71" s="12"/>
+      <c r="J71" s="12"/>
+      <c r="K71" s="12"/>
+      <c r="L71" s="12"/>
+      <c r="M71" s="12"/>
+      <c r="N71" s="12"/>
+      <c r="O71" s="12"/>
+      <c r="P71" s="12"/>
+      <c r="Q71" s="12"/>
+      <c r="R71" s="12"/>
+      <c r="S71" s="12"/>
+      <c r="T71" s="12"/>
+      <c r="U71" s="12"/>
+      <c r="V71" s="12"/>
+      <c r="W71" s="12"/>
+      <c r="X71" s="12"/>
+    </row>
+    <row r="72" spans="1:24">
+      <c r="A72" s="12"/>
+      <c r="B72" s="7"/>
+      <c r="C72" s="13"/>
+      <c r="D72" s="12"/>
+      <c r="E72" s="12"/>
+      <c r="F72" s="12"/>
+      <c r="G72" s="12"/>
+      <c r="H72" s="12"/>
+      <c r="I72" s="12"/>
+      <c r="J72" s="12"/>
+      <c r="K72" s="12"/>
+      <c r="L72" s="12"/>
+      <c r="M72" s="12"/>
+      <c r="N72" s="12"/>
+      <c r="O72" s="12"/>
+      <c r="P72" s="12"/>
+      <c r="Q72" s="12"/>
+      <c r="R72" s="12"/>
+      <c r="S72" s="12"/>
+      <c r="T72" s="12"/>
+      <c r="U72" s="12"/>
+      <c r="V72" s="12"/>
+      <c r="W72" s="12"/>
+      <c r="X72" s="12"/>
+    </row>
+    <row r="73" spans="1:24">
+      <c r="A73" s="12"/>
+      <c r="B73" s="7"/>
+      <c r="C73" s="13"/>
+      <c r="D73" s="12"/>
+      <c r="E73" s="12"/>
+      <c r="F73" s="12"/>
+      <c r="G73" s="12"/>
+      <c r="H73" s="12"/>
+      <c r="I73" s="12"/>
+      <c r="J73" s="12"/>
+      <c r="K73" s="12"/>
+      <c r="L73" s="12"/>
+      <c r="M73" s="12"/>
+      <c r="N73" s="12"/>
+      <c r="O73" s="12"/>
+      <c r="P73" s="12"/>
+      <c r="Q73" s="12"/>
+      <c r="R73" s="12"/>
+      <c r="S73" s="12"/>
+      <c r="T73" s="12"/>
+      <c r="U73" s="12"/>
+      <c r="V73" s="12"/>
+      <c r="W73" s="12"/>
+      <c r="X73" s="12"/>
+    </row>
+    <row r="74" spans="1:24">
+      <c r="A74" s="12"/>
+      <c r="B74" s="7"/>
+      <c r="C74" s="13"/>
+      <c r="D74" s="12"/>
+      <c r="E74" s="12"/>
+      <c r="F74" s="12"/>
+      <c r="G74" s="12"/>
+      <c r="H74" s="12"/>
+      <c r="I74" s="12"/>
+      <c r="J74" s="12"/>
+      <c r="K74" s="12"/>
+      <c r="L74" s="12"/>
+      <c r="M74" s="12"/>
+      <c r="N74" s="12"/>
+      <c r="O74" s="12"/>
+      <c r="P74" s="12"/>
+      <c r="Q74" s="12"/>
+      <c r="R74" s="12"/>
+      <c r="S74" s="12"/>
+      <c r="T74" s="12"/>
+      <c r="U74" s="12"/>
+      <c r="V74" s="12"/>
+      <c r="W74" s="12"/>
+      <c r="X74" s="12"/>
+    </row>
+    <row r="75" spans="1:24">
+      <c r="A75" s="12"/>
+      <c r="B75" s="7"/>
+      <c r="C75" s="13"/>
+      <c r="D75" s="12"/>
+      <c r="E75" s="12"/>
+      <c r="F75" s="12"/>
+      <c r="G75" s="12"/>
+      <c r="H75" s="12"/>
+      <c r="I75" s="12"/>
+      <c r="J75" s="12"/>
+      <c r="K75" s="12"/>
+      <c r="L75" s="12"/>
+      <c r="M75" s="12"/>
+      <c r="N75" s="12"/>
+      <c r="O75" s="12"/>
+      <c r="P75" s="12"/>
+      <c r="Q75" s="12"/>
+      <c r="R75" s="12"/>
+      <c r="S75" s="12"/>
+      <c r="T75" s="12"/>
+      <c r="U75" s="12"/>
+      <c r="V75" s="12"/>
+      <c r="W75" s="12"/>
+      <c r="X75" s="12"/>
+    </row>
+    <row r="76" spans="1:24">
+      <c r="A76" s="12"/>
+      <c r="B76" s="7"/>
+      <c r="C76" s="13"/>
+      <c r="D76" s="12"/>
+      <c r="E76" s="12"/>
+      <c r="F76" s="12"/>
+      <c r="G76" s="12"/>
+      <c r="H76" s="12"/>
+      <c r="I76" s="12"/>
+      <c r="J76" s="12"/>
+      <c r="K76" s="12"/>
+      <c r="L76" s="12"/>
+      <c r="M76" s="12"/>
+      <c r="N76" s="12"/>
+      <c r="O76" s="12"/>
+      <c r="P76" s="12"/>
+      <c r="Q76" s="12"/>
+      <c r="R76" s="12"/>
+      <c r="S76" s="12"/>
+      <c r="T76" s="12"/>
+      <c r="U76" s="12"/>
+      <c r="V76" s="12"/>
+      <c r="W76" s="12"/>
+      <c r="X76" s="12"/>
     </row>
     <row r="77" spans="1:24">
-      <c r="A77" s="1"/>
-      <c r="B77" s="2"/>
-      <c r="C77" s="3"/>
-      <c r="D77" s="1"/>
-      <c r="E77" s="1"/>
-      <c r="F77" s="1"/>
-      <c r="G77" s="1"/>
-      <c r="H77" s="1"/>
-      <c r="I77" s="1"/>
-      <c r="J77" s="1"/>
-      <c r="K77" s="1"/>
-      <c r="L77" s="1"/>
-      <c r="M77" s="1"/>
-      <c r="N77" s="1"/>
-      <c r="O77" s="1"/>
-      <c r="P77" s="1"/>
-      <c r="Q77" s="1"/>
-      <c r="R77" s="1"/>
-      <c r="S77" s="1"/>
-      <c r="T77" s="1"/>
-      <c r="U77" s="1"/>
-      <c r="V77" s="1"/>
-      <c r="W77" s="1"/>
-      <c r="X77" s="1"/>
+      <c r="A77" s="12"/>
+      <c r="B77" s="7"/>
+      <c r="C77" s="13"/>
+      <c r="D77" s="12"/>
+      <c r="E77" s="12"/>
+      <c r="F77" s="12"/>
+      <c r="G77" s="12"/>
+      <c r="H77" s="12"/>
+      <c r="I77" s="12"/>
+      <c r="J77" s="12"/>
+      <c r="K77" s="12"/>
+      <c r="L77" s="12"/>
+      <c r="M77" s="12"/>
+      <c r="N77" s="12"/>
+      <c r="O77" s="12"/>
+      <c r="P77" s="12"/>
+      <c r="Q77" s="12"/>
+      <c r="R77" s="12"/>
+      <c r="S77" s="12"/>
+      <c r="T77" s="12"/>
+      <c r="U77" s="12"/>
+      <c r="V77" s="12"/>
+      <c r="W77" s="12"/>
+      <c r="X77" s="12"/>
     </row>
     <row r="78" spans="1:24">
-      <c r="A78" s="1"/>
-      <c r="B78" s="2"/>
-      <c r="C78" s="3"/>
-      <c r="D78" s="1"/>
-      <c r="E78" s="1"/>
-      <c r="F78" s="1"/>
-      <c r="G78" s="1"/>
-      <c r="H78" s="1"/>
-      <c r="I78" s="1"/>
-      <c r="J78" s="1"/>
-      <c r="K78" s="1"/>
-      <c r="L78" s="1"/>
-      <c r="M78" s="1"/>
-      <c r="N78" s="1"/>
-      <c r="O78" s="1"/>
-      <c r="P78" s="1"/>
-      <c r="Q78" s="1"/>
-      <c r="R78" s="1"/>
-      <c r="S78" s="1"/>
-      <c r="T78" s="1"/>
-      <c r="U78" s="1"/>
-      <c r="V78" s="1"/>
-      <c r="W78" s="1"/>
-      <c r="X78" s="1"/>
+      <c r="A78" s="12"/>
+      <c r="B78" s="7"/>
+      <c r="C78" s="13"/>
+      <c r="D78" s="12"/>
+      <c r="E78" s="12"/>
+      <c r="F78" s="12"/>
+      <c r="G78" s="12"/>
+      <c r="H78" s="12"/>
+      <c r="I78" s="12"/>
+      <c r="J78" s="12"/>
+      <c r="K78" s="12"/>
+      <c r="L78" s="12"/>
+      <c r="M78" s="12"/>
+      <c r="N78" s="12"/>
+      <c r="O78" s="12"/>
+      <c r="P78" s="12"/>
+      <c r="Q78" s="12"/>
+      <c r="R78" s="12"/>
+      <c r="S78" s="12"/>
+      <c r="T78" s="12"/>
+      <c r="U78" s="12"/>
+      <c r="V78" s="12"/>
+      <c r="W78" s="12"/>
+      <c r="X78" s="12"/>
     </row>
     <row r="79" spans="1:24">
-      <c r="A79" s="1"/>
-      <c r="B79" s="2"/>
-      <c r="C79" s="3"/>
-      <c r="D79" s="1"/>
-      <c r="E79" s="1"/>
-      <c r="F79" s="1"/>
-      <c r="G79" s="1"/>
-      <c r="H79" s="1"/>
-      <c r="I79" s="1"/>
-      <c r="J79" s="1"/>
-      <c r="K79" s="1"/>
-      <c r="L79" s="1"/>
-      <c r="M79" s="1"/>
-      <c r="N79" s="1"/>
-      <c r="O79" s="1"/>
-      <c r="P79" s="1"/>
-      <c r="Q79" s="1"/>
-      <c r="R79" s="1"/>
-      <c r="S79" s="1"/>
-      <c r="T79" s="1"/>
-      <c r="U79" s="1"/>
-      <c r="V79" s="1"/>
-      <c r="W79" s="1"/>
-      <c r="X79" s="1"/>
+      <c r="A79" s="12"/>
+      <c r="B79" s="7"/>
+      <c r="C79" s="13"/>
+      <c r="D79" s="12"/>
+      <c r="E79" s="12"/>
+      <c r="F79" s="12"/>
+      <c r="G79" s="12"/>
+      <c r="H79" s="12"/>
+      <c r="I79" s="12"/>
+      <c r="J79" s="12"/>
+      <c r="K79" s="12"/>
+      <c r="L79" s="12"/>
+      <c r="M79" s="12"/>
+      <c r="N79" s="12"/>
+      <c r="O79" s="12"/>
+      <c r="P79" s="12"/>
+      <c r="Q79" s="12"/>
+      <c r="R79" s="12"/>
+      <c r="S79" s="12"/>
+      <c r="T79" s="12"/>
+      <c r="U79" s="12"/>
+      <c r="V79" s="12"/>
+      <c r="W79" s="12"/>
+      <c r="X79" s="12"/>
     </row>
     <row r="80" spans="1:24">
-      <c r="A80" s="1"/>
-      <c r="B80" s="2"/>
-      <c r="C80" s="3"/>
-      <c r="D80" s="1"/>
-      <c r="E80" s="1"/>
-      <c r="F80" s="1"/>
-      <c r="G80" s="1"/>
-      <c r="H80" s="1"/>
-      <c r="I80" s="1"/>
-      <c r="J80" s="1"/>
-      <c r="K80" s="1"/>
-      <c r="L80" s="1"/>
-      <c r="M80" s="1"/>
-      <c r="N80" s="1"/>
-      <c r="O80" s="1"/>
-      <c r="P80" s="1"/>
-      <c r="Q80" s="1"/>
-      <c r="R80" s="1"/>
-      <c r="S80" s="1"/>
-      <c r="T80" s="1"/>
-      <c r="U80" s="1"/>
-      <c r="V80" s="1"/>
-      <c r="W80" s="1"/>
-      <c r="X80" s="1"/>
+      <c r="A80" s="12"/>
+      <c r="B80" s="7"/>
+      <c r="C80" s="13"/>
+      <c r="D80" s="12"/>
+      <c r="E80" s="12"/>
+      <c r="F80" s="12"/>
+      <c r="G80" s="12"/>
+      <c r="H80" s="12"/>
+      <c r="I80" s="12"/>
+      <c r="J80" s="12"/>
+      <c r="K80" s="12"/>
+      <c r="L80" s="12"/>
+      <c r="M80" s="12"/>
+      <c r="N80" s="12"/>
+      <c r="O80" s="12"/>
+      <c r="P80" s="12"/>
+      <c r="Q80" s="12"/>
+      <c r="R80" s="12"/>
+      <c r="S80" s="12"/>
+      <c r="T80" s="12"/>
+      <c r="U80" s="12"/>
+      <c r="V80" s="12"/>
+      <c r="W80" s="12"/>
+      <c r="X80" s="12"/>
     </row>
     <row r="81" spans="1:24">
-      <c r="A81" s="1"/>
-      <c r="B81" s="2"/>
-      <c r="C81" s="3"/>
-      <c r="D81" s="1"/>
-      <c r="E81" s="1"/>
-      <c r="F81" s="1"/>
-      <c r="G81" s="1"/>
-      <c r="H81" s="1"/>
-      <c r="I81" s="1"/>
-      <c r="J81" s="1"/>
-      <c r="K81" s="1"/>
-      <c r="L81" s="1"/>
-      <c r="M81" s="1"/>
-      <c r="N81" s="1"/>
-      <c r="O81" s="1"/>
-      <c r="P81" s="1"/>
-      <c r="Q81" s="1"/>
-      <c r="R81" s="1"/>
-      <c r="S81" s="1"/>
-      <c r="T81" s="1"/>
-      <c r="U81" s="1"/>
-      <c r="V81" s="1"/>
-      <c r="W81" s="1"/>
-      <c r="X81" s="1"/>
+      <c r="A81" s="12"/>
+      <c r="B81" s="7"/>
+      <c r="C81" s="13"/>
+      <c r="D81" s="12"/>
+      <c r="E81" s="12"/>
+      <c r="F81" s="12"/>
+      <c r="G81" s="12"/>
+      <c r="H81" s="12"/>
+      <c r="I81" s="12"/>
+      <c r="J81" s="12"/>
+      <c r="K81" s="12"/>
+      <c r="L81" s="12"/>
+      <c r="M81" s="12"/>
+      <c r="N81" s="12"/>
+      <c r="O81" s="12"/>
+      <c r="P81" s="12"/>
+      <c r="Q81" s="12"/>
+      <c r="R81" s="12"/>
+      <c r="S81" s="12"/>
+      <c r="T81" s="12"/>
+      <c r="U81" s="12"/>
+      <c r="V81" s="12"/>
+      <c r="W81" s="12"/>
+      <c r="X81" s="12"/>
     </row>
     <row r="82" spans="1:24">
-      <c r="A82" s="1"/>
-      <c r="B82" s="2"/>
-      <c r="C82" s="3"/>
-      <c r="D82" s="1"/>
-      <c r="E82" s="1"/>
-      <c r="F82" s="1"/>
-      <c r="G82" s="1"/>
-      <c r="H82" s="1"/>
-      <c r="I82" s="1"/>
-      <c r="J82" s="1"/>
-      <c r="K82" s="1"/>
-      <c r="L82" s="1"/>
-      <c r="M82" s="1"/>
-      <c r="N82" s="1"/>
-      <c r="O82" s="1"/>
-      <c r="P82" s="1"/>
-      <c r="Q82" s="1"/>
-      <c r="R82" s="1"/>
-      <c r="S82" s="1"/>
-      <c r="T82" s="1"/>
-      <c r="U82" s="1"/>
-      <c r="V82" s="1"/>
-      <c r="W82" s="1"/>
-      <c r="X82" s="1"/>
+      <c r="A82" s="12"/>
+      <c r="B82" s="7"/>
+      <c r="C82" s="13"/>
+      <c r="D82" s="12"/>
+      <c r="E82" s="12"/>
+      <c r="F82" s="12"/>
+      <c r="G82" s="12"/>
+      <c r="H82" s="12"/>
+      <c r="I82" s="12"/>
+      <c r="J82" s="12"/>
+      <c r="K82" s="12"/>
+      <c r="L82" s="12"/>
+      <c r="M82" s="12"/>
+      <c r="N82" s="12"/>
+      <c r="O82" s="12"/>
+      <c r="P82" s="12"/>
+      <c r="Q82" s="12"/>
+      <c r="R82" s="12"/>
+      <c r="S82" s="12"/>
+      <c r="T82" s="12"/>
+      <c r="U82" s="12"/>
+      <c r="V82" s="12"/>
+      <c r="W82" s="12"/>
+      <c r="X82" s="12"/>
     </row>
     <row r="83" spans="1:24">
       <c r="A83" s="12"/>
@@ -8474,633 +8265,10 @@
       <c r="W266" s="12"/>
       <c r="X266" s="12"/>
     </row>
-    <row r="267" spans="1:24">
-      <c r="A267" s="12"/>
-      <c r="B267" s="7"/>
-      <c r="C267" s="13"/>
-      <c r="D267" s="12"/>
-      <c r="E267" s="12"/>
-      <c r="F267" s="12"/>
-      <c r="G267" s="12"/>
-      <c r="H267" s="12"/>
-      <c r="I267" s="12"/>
-      <c r="J267" s="12"/>
-      <c r="K267" s="12"/>
-      <c r="L267" s="12"/>
-      <c r="M267" s="12"/>
-      <c r="N267" s="12"/>
-      <c r="O267" s="12"/>
-      <c r="P267" s="12"/>
-      <c r="Q267" s="12"/>
-      <c r="R267" s="12"/>
-      <c r="S267" s="12"/>
-      <c r="T267" s="12"/>
-      <c r="U267" s="12"/>
-      <c r="V267" s="12"/>
-      <c r="W267" s="12"/>
-      <c r="X267" s="12"/>
-    </row>
-    <row r="268" spans="1:24">
-      <c r="A268" s="12"/>
-      <c r="B268" s="7"/>
-      <c r="C268" s="13"/>
-      <c r="D268" s="12"/>
-      <c r="E268" s="12"/>
-      <c r="F268" s="12"/>
-      <c r="G268" s="12"/>
-      <c r="H268" s="12"/>
-      <c r="I268" s="12"/>
-      <c r="J268" s="12"/>
-      <c r="K268" s="12"/>
-      <c r="L268" s="12"/>
-      <c r="M268" s="12"/>
-      <c r="N268" s="12"/>
-      <c r="O268" s="12"/>
-      <c r="P268" s="12"/>
-      <c r="Q268" s="12"/>
-      <c r="R268" s="12"/>
-      <c r="S268" s="12"/>
-      <c r="T268" s="12"/>
-      <c r="U268" s="12"/>
-      <c r="V268" s="12"/>
-      <c r="W268" s="12"/>
-      <c r="X268" s="12"/>
-    </row>
-    <row r="269" spans="1:24">
-      <c r="A269" s="12"/>
-      <c r="B269" s="7"/>
-      <c r="C269" s="13"/>
-      <c r="D269" s="12"/>
-      <c r="E269" s="12"/>
-      <c r="F269" s="12"/>
-      <c r="G269" s="12"/>
-      <c r="H269" s="12"/>
-      <c r="I269" s="12"/>
-      <c r="J269" s="12"/>
-      <c r="K269" s="12"/>
-      <c r="L269" s="12"/>
-      <c r="M269" s="12"/>
-      <c r="N269" s="12"/>
-      <c r="O269" s="12"/>
-      <c r="P269" s="12"/>
-      <c r="Q269" s="12"/>
-      <c r="R269" s="12"/>
-      <c r="S269" s="12"/>
-      <c r="T269" s="12"/>
-      <c r="U269" s="12"/>
-      <c r="V269" s="12"/>
-      <c r="W269" s="12"/>
-      <c r="X269" s="12"/>
-    </row>
-    <row r="270" spans="1:24">
-      <c r="A270" s="12"/>
-      <c r="B270" s="7"/>
-      <c r="C270" s="13"/>
-      <c r="D270" s="12"/>
-      <c r="E270" s="12"/>
-      <c r="F270" s="12"/>
-      <c r="G270" s="12"/>
-      <c r="H270" s="12"/>
-      <c r="I270" s="12"/>
-      <c r="J270" s="12"/>
-      <c r="K270" s="12"/>
-      <c r="L270" s="12"/>
-      <c r="M270" s="12"/>
-      <c r="N270" s="12"/>
-      <c r="O270" s="12"/>
-      <c r="P270" s="12"/>
-      <c r="Q270" s="12"/>
-      <c r="R270" s="12"/>
-      <c r="S270" s="12"/>
-      <c r="T270" s="12"/>
-      <c r="U270" s="12"/>
-      <c r="V270" s="12"/>
-      <c r="W270" s="12"/>
-      <c r="X270" s="12"/>
-    </row>
-    <row r="271" spans="1:24">
-      <c r="A271" s="12"/>
-      <c r="B271" s="7"/>
-      <c r="C271" s="13"/>
-      <c r="D271" s="12"/>
-      <c r="E271" s="12"/>
-      <c r="F271" s="12"/>
-      <c r="G271" s="12"/>
-      <c r="H271" s="12"/>
-      <c r="I271" s="12"/>
-      <c r="J271" s="12"/>
-      <c r="K271" s="12"/>
-      <c r="L271" s="12"/>
-      <c r="M271" s="12"/>
-      <c r="N271" s="12"/>
-      <c r="O271" s="12"/>
-      <c r="P271" s="12"/>
-      <c r="Q271" s="12"/>
-      <c r="R271" s="12"/>
-      <c r="S271" s="12"/>
-      <c r="T271" s="12"/>
-      <c r="U271" s="12"/>
-      <c r="V271" s="12"/>
-      <c r="W271" s="12"/>
-      <c r="X271" s="12"/>
-    </row>
-    <row r="272" spans="1:24">
-      <c r="A272" s="12"/>
-      <c r="B272" s="7"/>
-      <c r="C272" s="13"/>
-      <c r="D272" s="12"/>
-      <c r="E272" s="12"/>
-      <c r="F272" s="12"/>
-      <c r="G272" s="12"/>
-      <c r="H272" s="12"/>
-      <c r="I272" s="12"/>
-      <c r="J272" s="12"/>
-      <c r="K272" s="12"/>
-      <c r="L272" s="12"/>
-      <c r="M272" s="12"/>
-      <c r="N272" s="12"/>
-      <c r="O272" s="12"/>
-      <c r="P272" s="12"/>
-      <c r="Q272" s="12"/>
-      <c r="R272" s="12"/>
-      <c r="S272" s="12"/>
-      <c r="T272" s="12"/>
-      <c r="U272" s="12"/>
-      <c r="V272" s="12"/>
-      <c r="W272" s="12"/>
-      <c r="X272" s="12"/>
-    </row>
-    <row r="273" spans="1:24">
-      <c r="A273" s="12"/>
-      <c r="B273" s="7"/>
-      <c r="C273" s="13"/>
-      <c r="D273" s="12"/>
-      <c r="E273" s="12"/>
-      <c r="F273" s="12"/>
-      <c r="G273" s="12"/>
-      <c r="H273" s="12"/>
-      <c r="I273" s="12"/>
-      <c r="J273" s="12"/>
-      <c r="K273" s="12"/>
-      <c r="L273" s="12"/>
-      <c r="M273" s="12"/>
-      <c r="N273" s="12"/>
-      <c r="O273" s="12"/>
-      <c r="P273" s="12"/>
-      <c r="Q273" s="12"/>
-      <c r="R273" s="12"/>
-      <c r="S273" s="12"/>
-      <c r="T273" s="12"/>
-      <c r="U273" s="12"/>
-      <c r="V273" s="12"/>
-      <c r="W273" s="12"/>
-      <c r="X273" s="12"/>
-    </row>
-    <row r="274" spans="1:24">
-      <c r="A274" s="12"/>
-      <c r="B274" s="7"/>
-      <c r="C274" s="13"/>
-      <c r="D274" s="12"/>
-      <c r="E274" s="12"/>
-      <c r="F274" s="12"/>
-      <c r="G274" s="12"/>
-      <c r="H274" s="12"/>
-      <c r="I274" s="12"/>
-      <c r="J274" s="12"/>
-      <c r="K274" s="12"/>
-      <c r="L274" s="12"/>
-      <c r="M274" s="12"/>
-      <c r="N274" s="12"/>
-      <c r="O274" s="12"/>
-      <c r="P274" s="12"/>
-      <c r="Q274" s="12"/>
-      <c r="R274" s="12"/>
-      <c r="S274" s="12"/>
-      <c r="T274" s="12"/>
-      <c r="U274" s="12"/>
-      <c r="V274" s="12"/>
-      <c r="W274" s="12"/>
-      <c r="X274" s="12"/>
-    </row>
-    <row r="275" spans="1:24">
-      <c r="A275" s="12"/>
-      <c r="B275" s="7"/>
-      <c r="C275" s="13"/>
-      <c r="D275" s="12"/>
-      <c r="E275" s="12"/>
-      <c r="F275" s="12"/>
-      <c r="G275" s="12"/>
-      <c r="H275" s="12"/>
-      <c r="I275" s="12"/>
-      <c r="J275" s="12"/>
-      <c r="K275" s="12"/>
-      <c r="L275" s="12"/>
-      <c r="M275" s="12"/>
-      <c r="N275" s="12"/>
-      <c r="O275" s="12"/>
-      <c r="P275" s="12"/>
-      <c r="Q275" s="12"/>
-      <c r="R275" s="12"/>
-      <c r="S275" s="12"/>
-      <c r="T275" s="12"/>
-      <c r="U275" s="12"/>
-      <c r="V275" s="12"/>
-      <c r="W275" s="12"/>
-      <c r="X275" s="12"/>
-    </row>
-    <row r="276" spans="1:24">
-      <c r="A276" s="12"/>
-      <c r="B276" s="7"/>
-      <c r="C276" s="13"/>
-      <c r="D276" s="12"/>
-      <c r="E276" s="12"/>
-      <c r="F276" s="12"/>
-      <c r="G276" s="12"/>
-      <c r="H276" s="12"/>
-      <c r="I276" s="12"/>
-      <c r="J276" s="12"/>
-      <c r="K276" s="12"/>
-      <c r="L276" s="12"/>
-      <c r="M276" s="12"/>
-      <c r="N276" s="12"/>
-      <c r="O276" s="12"/>
-      <c r="P276" s="12"/>
-      <c r="Q276" s="12"/>
-      <c r="R276" s="12"/>
-      <c r="S276" s="12"/>
-      <c r="T276" s="12"/>
-      <c r="U276" s="12"/>
-      <c r="V276" s="12"/>
-      <c r="W276" s="12"/>
-      <c r="X276" s="12"/>
-    </row>
-    <row r="277" spans="1:24">
-      <c r="A277" s="12"/>
-      <c r="B277" s="7"/>
-      <c r="C277" s="13"/>
-      <c r="D277" s="12"/>
-      <c r="E277" s="12"/>
-      <c r="F277" s="12"/>
-      <c r="G277" s="12"/>
-      <c r="H277" s="12"/>
-      <c r="I277" s="12"/>
-      <c r="J277" s="12"/>
-      <c r="K277" s="12"/>
-      <c r="L277" s="12"/>
-      <c r="M277" s="12"/>
-      <c r="N277" s="12"/>
-      <c r="O277" s="12"/>
-      <c r="P277" s="12"/>
-      <c r="Q277" s="12"/>
-      <c r="R277" s="12"/>
-      <c r="S277" s="12"/>
-      <c r="T277" s="12"/>
-      <c r="U277" s="12"/>
-      <c r="V277" s="12"/>
-      <c r="W277" s="12"/>
-      <c r="X277" s="12"/>
-    </row>
-    <row r="278" spans="1:24">
-      <c r="A278" s="12"/>
-      <c r="B278" s="7"/>
-      <c r="C278" s="13"/>
-      <c r="D278" s="12"/>
-      <c r="E278" s="12"/>
-      <c r="F278" s="12"/>
-      <c r="G278" s="12"/>
-      <c r="H278" s="12"/>
-      <c r="I278" s="12"/>
-      <c r="J278" s="12"/>
-      <c r="K278" s="12"/>
-      <c r="L278" s="12"/>
-      <c r="M278" s="12"/>
-      <c r="N278" s="12"/>
-      <c r="O278" s="12"/>
-      <c r="P278" s="12"/>
-      <c r="Q278" s="12"/>
-      <c r="R278" s="12"/>
-      <c r="S278" s="12"/>
-      <c r="T278" s="12"/>
-      <c r="U278" s="12"/>
-      <c r="V278" s="12"/>
-      <c r="W278" s="12"/>
-      <c r="X278" s="12"/>
-    </row>
-    <row r="279" spans="1:24">
-      <c r="A279" s="12"/>
-      <c r="B279" s="7"/>
-      <c r="C279" s="13"/>
-      <c r="D279" s="12"/>
-      <c r="E279" s="12"/>
-      <c r="F279" s="12"/>
-      <c r="G279" s="12"/>
-      <c r="H279" s="12"/>
-      <c r="I279" s="12"/>
-      <c r="J279" s="12"/>
-      <c r="K279" s="12"/>
-      <c r="L279" s="12"/>
-      <c r="M279" s="12"/>
-      <c r="N279" s="12"/>
-      <c r="O279" s="12"/>
-      <c r="P279" s="12"/>
-      <c r="Q279" s="12"/>
-      <c r="R279" s="12"/>
-      <c r="S279" s="12"/>
-      <c r="T279" s="12"/>
-      <c r="U279" s="12"/>
-      <c r="V279" s="12"/>
-      <c r="W279" s="12"/>
-      <c r="X279" s="12"/>
-    </row>
-    <row r="280" spans="1:24">
-      <c r="A280" s="12"/>
-      <c r="B280" s="7"/>
-      <c r="C280" s="13"/>
-      <c r="D280" s="12"/>
-      <c r="E280" s="12"/>
-      <c r="F280" s="12"/>
-      <c r="G280" s="12"/>
-      <c r="H280" s="12"/>
-      <c r="I280" s="12"/>
-      <c r="J280" s="12"/>
-      <c r="K280" s="12"/>
-      <c r="L280" s="12"/>
-      <c r="M280" s="12"/>
-      <c r="N280" s="12"/>
-      <c r="O280" s="12"/>
-      <c r="P280" s="12"/>
-      <c r="Q280" s="12"/>
-      <c r="R280" s="12"/>
-      <c r="S280" s="12"/>
-      <c r="T280" s="12"/>
-      <c r="U280" s="12"/>
-      <c r="V280" s="12"/>
-      <c r="W280" s="12"/>
-      <c r="X280" s="12"/>
-    </row>
-    <row r="281" spans="1:24">
-      <c r="A281" s="12"/>
-      <c r="B281" s="7"/>
-      <c r="C281" s="13"/>
-      <c r="D281" s="12"/>
-      <c r="E281" s="12"/>
-      <c r="F281" s="12"/>
-      <c r="G281" s="12"/>
-      <c r="H281" s="12"/>
-      <c r="I281" s="12"/>
-      <c r="J281" s="12"/>
-      <c r="K281" s="12"/>
-      <c r="L281" s="12"/>
-      <c r="M281" s="12"/>
-      <c r="N281" s="12"/>
-      <c r="O281" s="12"/>
-      <c r="P281" s="12"/>
-      <c r="Q281" s="12"/>
-      <c r="R281" s="12"/>
-      <c r="S281" s="12"/>
-      <c r="T281" s="12"/>
-      <c r="U281" s="12"/>
-      <c r="V281" s="12"/>
-      <c r="W281" s="12"/>
-      <c r="X281" s="12"/>
-    </row>
-    <row r="282" spans="1:24">
-      <c r="A282" s="12"/>
-      <c r="B282" s="7"/>
-      <c r="C282" s="13"/>
-      <c r="D282" s="12"/>
-      <c r="E282" s="12"/>
-      <c r="F282" s="12"/>
-      <c r="G282" s="12"/>
-      <c r="H282" s="12"/>
-      <c r="I282" s="12"/>
-      <c r="J282" s="12"/>
-      <c r="K282" s="12"/>
-      <c r="L282" s="12"/>
-      <c r="M282" s="12"/>
-      <c r="N282" s="12"/>
-      <c r="O282" s="12"/>
-      <c r="P282" s="12"/>
-      <c r="Q282" s="12"/>
-      <c r="R282" s="12"/>
-      <c r="S282" s="12"/>
-      <c r="T282" s="12"/>
-      <c r="U282" s="12"/>
-      <c r="V282" s="12"/>
-      <c r="W282" s="12"/>
-      <c r="X282" s="12"/>
-    </row>
-    <row r="283" spans="1:24">
-      <c r="A283" s="12"/>
-      <c r="B283" s="7"/>
-      <c r="C283" s="13"/>
-      <c r="D283" s="12"/>
-      <c r="E283" s="12"/>
-      <c r="F283" s="12"/>
-      <c r="G283" s="12"/>
-      <c r="H283" s="12"/>
-      <c r="I283" s="12"/>
-      <c r="J283" s="12"/>
-      <c r="K283" s="12"/>
-      <c r="L283" s="12"/>
-      <c r="M283" s="12"/>
-      <c r="N283" s="12"/>
-      <c r="O283" s="12"/>
-      <c r="P283" s="12"/>
-      <c r="Q283" s="12"/>
-      <c r="R283" s="12"/>
-      <c r="S283" s="12"/>
-      <c r="T283" s="12"/>
-      <c r="U283" s="12"/>
-      <c r="V283" s="12"/>
-      <c r="W283" s="12"/>
-      <c r="X283" s="12"/>
-    </row>
-    <row r="284" spans="1:24">
-      <c r="A284" s="12"/>
-      <c r="B284" s="7"/>
-      <c r="C284" s="13"/>
-      <c r="D284" s="12"/>
-      <c r="E284" s="12"/>
-      <c r="F284" s="12"/>
-      <c r="G284" s="12"/>
-      <c r="H284" s="12"/>
-      <c r="I284" s="12"/>
-      <c r="J284" s="12"/>
-      <c r="K284" s="12"/>
-      <c r="L284" s="12"/>
-      <c r="M284" s="12"/>
-      <c r="N284" s="12"/>
-      <c r="O284" s="12"/>
-      <c r="P284" s="12"/>
-      <c r="Q284" s="12"/>
-      <c r="R284" s="12"/>
-      <c r="S284" s="12"/>
-      <c r="T284" s="12"/>
-      <c r="U284" s="12"/>
-      <c r="V284" s="12"/>
-      <c r="W284" s="12"/>
-      <c r="X284" s="12"/>
-    </row>
-    <row r="285" spans="1:24">
-      <c r="A285" s="12"/>
-      <c r="B285" s="7"/>
-      <c r="C285" s="13"/>
-      <c r="D285" s="12"/>
-      <c r="E285" s="12"/>
-      <c r="F285" s="12"/>
-      <c r="G285" s="12"/>
-      <c r="H285" s="12"/>
-      <c r="I285" s="12"/>
-      <c r="J285" s="12"/>
-      <c r="K285" s="12"/>
-      <c r="L285" s="12"/>
-      <c r="M285" s="12"/>
-      <c r="N285" s="12"/>
-      <c r="O285" s="12"/>
-      <c r="P285" s="12"/>
-      <c r="Q285" s="12"/>
-      <c r="R285" s="12"/>
-      <c r="S285" s="12"/>
-      <c r="T285" s="12"/>
-      <c r="U285" s="12"/>
-      <c r="V285" s="12"/>
-      <c r="W285" s="12"/>
-      <c r="X285" s="12"/>
-    </row>
-    <row r="286" spans="1:24">
-      <c r="A286" s="12"/>
-      <c r="B286" s="7"/>
-      <c r="C286" s="13"/>
-      <c r="D286" s="12"/>
-      <c r="E286" s="12"/>
-      <c r="F286" s="12"/>
-      <c r="G286" s="12"/>
-      <c r="H286" s="12"/>
-      <c r="I286" s="12"/>
-      <c r="J286" s="12"/>
-      <c r="K286" s="12"/>
-      <c r="L286" s="12"/>
-      <c r="M286" s="12"/>
-      <c r="N286" s="12"/>
-      <c r="O286" s="12"/>
-      <c r="P286" s="12"/>
-      <c r="Q286" s="12"/>
-      <c r="R286" s="12"/>
-      <c r="S286" s="12"/>
-      <c r="T286" s="12"/>
-      <c r="U286" s="12"/>
-      <c r="V286" s="12"/>
-      <c r="W286" s="12"/>
-      <c r="X286" s="12"/>
-    </row>
-    <row r="287" spans="1:24">
-      <c r="A287" s="12"/>
-      <c r="B287" s="7"/>
-      <c r="C287" s="13"/>
-      <c r="D287" s="12"/>
-      <c r="E287" s="12"/>
-      <c r="F287" s="12"/>
-      <c r="G287" s="12"/>
-      <c r="H287" s="12"/>
-      <c r="I287" s="12"/>
-      <c r="J287" s="12"/>
-      <c r="K287" s="12"/>
-      <c r="L287" s="12"/>
-      <c r="M287" s="12"/>
-      <c r="N287" s="12"/>
-      <c r="O287" s="12"/>
-      <c r="P287" s="12"/>
-      <c r="Q287" s="12"/>
-      <c r="R287" s="12"/>
-      <c r="S287" s="12"/>
-      <c r="T287" s="12"/>
-      <c r="U287" s="12"/>
-      <c r="V287" s="12"/>
-      <c r="W287" s="12"/>
-      <c r="X287" s="12"/>
-    </row>
-    <row r="288" spans="1:24">
-      <c r="A288" s="12"/>
-      <c r="B288" s="7"/>
-      <c r="C288" s="13"/>
-      <c r="D288" s="12"/>
-      <c r="E288" s="12"/>
-      <c r="F288" s="12"/>
-      <c r="G288" s="12"/>
-      <c r="H288" s="12"/>
-      <c r="I288" s="12"/>
-      <c r="J288" s="12"/>
-      <c r="K288" s="12"/>
-      <c r="L288" s="12"/>
-      <c r="M288" s="12"/>
-      <c r="N288" s="12"/>
-      <c r="O288" s="12"/>
-      <c r="P288" s="12"/>
-      <c r="Q288" s="12"/>
-      <c r="R288" s="12"/>
-      <c r="S288" s="12"/>
-      <c r="T288" s="12"/>
-      <c r="U288" s="12"/>
-      <c r="V288" s="12"/>
-      <c r="W288" s="12"/>
-      <c r="X288" s="12"/>
-    </row>
-    <row r="289" spans="1:24">
-      <c r="A289" s="12"/>
-      <c r="B289" s="7"/>
-      <c r="C289" s="13"/>
-      <c r="D289" s="12"/>
-      <c r="E289" s="12"/>
-      <c r="F289" s="12"/>
-      <c r="G289" s="12"/>
-      <c r="H289" s="12"/>
-      <c r="I289" s="12"/>
-      <c r="J289" s="12"/>
-      <c r="K289" s="12"/>
-      <c r="L289" s="12"/>
-      <c r="M289" s="12"/>
-      <c r="N289" s="12"/>
-      <c r="O289" s="12"/>
-      <c r="P289" s="12"/>
-      <c r="Q289" s="12"/>
-      <c r="R289" s="12"/>
-      <c r="S289" s="12"/>
-      <c r="T289" s="12"/>
-      <c r="U289" s="12"/>
-      <c r="V289" s="12"/>
-      <c r="W289" s="12"/>
-      <c r="X289" s="12"/>
-    </row>
-    <row r="290" spans="1:24">
-      <c r="A290" s="12"/>
-      <c r="B290" s="7"/>
-      <c r="C290" s="13"/>
-      <c r="D290" s="12"/>
-      <c r="E290" s="12"/>
-      <c r="F290" s="12"/>
-      <c r="G290" s="12"/>
-      <c r="H290" s="12"/>
-      <c r="I290" s="12"/>
-      <c r="J290" s="12"/>
-      <c r="K290" s="12"/>
-      <c r="L290" s="12"/>
-      <c r="M290" s="12"/>
-      <c r="N290" s="12"/>
-      <c r="O290" s="12"/>
-      <c r="P290" s="12"/>
-      <c r="Q290" s="12"/>
-      <c r="R290" s="12"/>
-      <c r="S290" s="12"/>
-      <c r="T290" s="12"/>
-      <c r="U290" s="12"/>
-      <c r="V290" s="12"/>
-      <c r="W290" s="12"/>
-      <c r="X290" s="12"/>
-    </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Ajuste adicion items plantilla dinamica y excel
</commit_message>
<xml_diff>
--- a/Assets/Plantillas/InstructivoPlantillaCargue.xlsx
+++ b/Assets/Plantillas/InstructivoPlantillaCargue.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr codeName="ThisWorkbook" hidePivotFieldList="1" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/72c68232ab824a52/Omar Akon Personal/Proyectos OAG/Bufins Web/Common/Adicionales/Plantilla cargue/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/72c68232ab824a52/Omar Akon Personal/Proyectos OAG/Bufins Web/Bufins principal web/bufinscustomers/Assets/Plantillas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="47" documentId="13_ncr:1_{028B1B36-2557-4057-A3FA-7676B7B3B9C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F915F77B-D69B-4721-8526-704C91356302}"/>
+  <xr:revisionPtr revIDLastSave="58" documentId="13_ncr:1_{028B1B36-2557-4057-A3FA-7676B7B3B9C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5EFA452F-25EA-4887-A568-C62417F7C593}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="598" xr2:uid="{FA4E9C0C-F0DD-43A6-9F82-B69A727F5A7D}"/>
   </bookViews>
@@ -70,7 +70,7 @@
     <definedName name="wrn.Informe._.Consolidado." hidden="1">{#N/A,#N/A,FALSE,"P o G";#N/A,#N/A,FALSE,"BALANCE";#N/A,#N/A,FALSE,"Indicadores";#N/A,#N/A,FALSE,"Capital Trab. (2)";#N/A,#N/A,FALSE,"Camb. Sit. Financ. (2)";#N/A,#N/A,FALSE,"ROTABCIUD"}</definedName>
     <definedName name="wrn.Junta._.Principal." hidden="1">{#N/A,#N/A,FALSE,"VENTAS";#N/A,#N/A,FALSE,"U. BRUTA";#N/A,#N/A,FALSE,"G. PERSONAL";#N/A,#N/A,FALSE,"G. OPERACION";#N/A,#N/A,FALSE,"G. DEPYAM";#N/A,#N/A,FALSE,"INGRESOS";#N/A,#N/A,FALSE,"G.o P.1";#N/A,#N/A,FALSE,"3%Informe Junta";#N/A,#N/A,FALSE,"P Y G (2)";#N/A,#N/A,FALSE,"CART. PROV.";#N/A,#N/A,FALSE,"Usecmes";#N/A,#N/A,FALSE,"Usecacu"}</definedName>
   </definedNames>
-  <calcPr calcId="191029" calcMode="autoNoTable" concurrentCalc="0"/>
+  <calcPr calcId="191029" calcMode="autoNoTable" iterate="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -111,7 +111,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="59">
   <si>
     <t>GASTOS FIJOS</t>
   </si>
@@ -296,6 +296,12 @@
   </si>
   <si>
     <t>Aplican las mismas instrucciones de la hoja Z_BalancePrueba a 4 dígitos del PUC, para las cuentas de activos y pasivos que deben calsificarse como de carácter corriente y no corriente</t>
+  </si>
+  <si>
+    <t>Es indispensable que en diciembre se cierren todas las cuentas temporales</t>
+  </si>
+  <si>
+    <t>Es indispensable que los resultados del mes estén registrados en la cuenta 36</t>
   </si>
 </sst>
 </file>
@@ -1236,7 +1242,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B746BB9-28D1-4089-9539-F175A9784447}">
-  <dimension ref="A1:X266"/>
+  <dimension ref="A1:X268"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="3.7109375" style="4" customWidth="1"/>
@@ -1713,8 +1719,12 @@
     </row>
     <row r="17" spans="1:24" ht="18">
       <c r="A17" s="1"/>
-      <c r="B17" s="10"/>
-      <c r="C17" s="3"/>
+      <c r="B17" s="10">
+        <v>11</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>58</v>
+      </c>
       <c r="D17" s="1"/>
       <c r="E17" s="1"/>
       <c r="F17" s="1"/>
@@ -1739,9 +1749,11 @@
     </row>
     <row r="18" spans="1:24" ht="18">
       <c r="A18" s="1"/>
-      <c r="B18" s="10"/>
-      <c r="C18" s="9" t="s">
-        <v>29</v>
+      <c r="B18" s="10">
+        <v>12</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>57</v>
       </c>
       <c r="D18" s="1"/>
       <c r="E18" s="1"/>
@@ -1765,14 +1777,10 @@
       <c r="W18" s="1"/>
       <c r="X18" s="1"/>
     </row>
-    <row r="19" spans="1:24" ht="15">
+    <row r="19" spans="1:24" ht="18">
       <c r="A19" s="1"/>
-      <c r="B19" s="11" t="s">
-        <v>9</v>
-      </c>
-      <c r="C19" s="3" t="s">
-        <v>16</v>
-      </c>
+      <c r="B19" s="10"/>
+      <c r="C19" s="3"/>
       <c r="D19" s="1"/>
       <c r="E19" s="1"/>
       <c r="F19" s="1"/>
@@ -1795,11 +1803,11 @@
       <c r="W19" s="1"/>
       <c r="X19" s="1"/>
     </row>
-    <row r="20" spans="1:24" ht="15">
+    <row r="20" spans="1:24" ht="18">
       <c r="A20" s="1"/>
-      <c r="B20" s="11"/>
-      <c r="C20" s="3" t="s">
-        <v>14</v>
+      <c r="B20" s="10"/>
+      <c r="C20" s="9" t="s">
+        <v>29</v>
       </c>
       <c r="D20" s="1"/>
       <c r="E20" s="1"/>
@@ -1825,9 +1833,11 @@
     </row>
     <row r="21" spans="1:24" ht="15">
       <c r="A21" s="1"/>
-      <c r="B21" s="11"/>
+      <c r="B21" s="11" t="s">
+        <v>9</v>
+      </c>
       <c r="C21" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D21" s="1"/>
       <c r="E21" s="1"/>
@@ -1851,11 +1861,11 @@
       <c r="W21" s="1"/>
       <c r="X21" s="1"/>
     </row>
-    <row r="22" spans="1:24" ht="28.5">
+    <row r="22" spans="1:24" ht="15">
       <c r="A22" s="1"/>
       <c r="B22" s="11"/>
       <c r="C22" s="3" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="D22" s="1"/>
       <c r="E22" s="1"/>
@@ -1883,7 +1893,7 @@
       <c r="A23" s="1"/>
       <c r="B23" s="11"/>
       <c r="C23" s="3" t="s">
-        <v>53</v>
+        <v>15</v>
       </c>
       <c r="D23" s="1"/>
       <c r="E23" s="1"/>
@@ -1909,11 +1919,9 @@
     </row>
     <row r="24" spans="1:24" ht="28.5">
       <c r="A24" s="1"/>
-      <c r="B24" s="11" t="s">
-        <v>10</v>
-      </c>
+      <c r="B24" s="11"/>
       <c r="C24" s="3" t="s">
-        <v>56</v>
+        <v>19</v>
       </c>
       <c r="D24" s="1"/>
       <c r="E24" s="1"/>
@@ -1937,11 +1945,11 @@
       <c r="W24" s="1"/>
       <c r="X24" s="1"/>
     </row>
-    <row r="25" spans="1:24" ht="28.5">
+    <row r="25" spans="1:24" ht="15">
       <c r="A25" s="1"/>
       <c r="B25" s="11"/>
       <c r="C25" s="3" t="s">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="D25" s="1"/>
       <c r="E25" s="1"/>
@@ -1965,11 +1973,13 @@
       <c r="W25" s="1"/>
       <c r="X25" s="1"/>
     </row>
-    <row r="26" spans="1:24" ht="15">
+    <row r="26" spans="1:24" ht="28.5">
       <c r="A26" s="1"/>
-      <c r="B26" s="11"/>
+      <c r="B26" s="11" t="s">
+        <v>10</v>
+      </c>
       <c r="C26" s="3" t="s">
-        <v>33</v>
+        <v>56</v>
       </c>
       <c r="D26" s="1"/>
       <c r="E26" s="1"/>
@@ -1993,13 +2003,11 @@
       <c r="W26" s="1"/>
       <c r="X26" s="1"/>
     </row>
-    <row r="27" spans="1:24" ht="15">
+    <row r="27" spans="1:24" ht="28.5">
       <c r="A27" s="1"/>
-      <c r="B27" s="11" t="s">
-        <v>11</v>
-      </c>
+      <c r="B27" s="11"/>
       <c r="C27" s="3" t="s">
-        <v>17</v>
+        <v>46</v>
       </c>
       <c r="D27" s="1"/>
       <c r="E27" s="1"/>
@@ -2027,7 +2035,7 @@
       <c r="A28" s="1"/>
       <c r="B28" s="11"/>
       <c r="C28" s="3" t="s">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="D28" s="1"/>
       <c r="E28" s="1"/>
@@ -2053,9 +2061,11 @@
     </row>
     <row r="29" spans="1:24" ht="15">
       <c r="A29" s="1"/>
-      <c r="B29" s="11"/>
+      <c r="B29" s="11" t="s">
+        <v>11</v>
+      </c>
       <c r="C29" s="3" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D29" s="1"/>
       <c r="E29" s="1"/>
@@ -2083,7 +2093,7 @@
       <c r="A30" s="1"/>
       <c r="B30" s="11"/>
       <c r="C30" s="3" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="D30" s="1"/>
       <c r="E30" s="1"/>
@@ -2107,11 +2117,11 @@
       <c r="W30" s="1"/>
       <c r="X30" s="1"/>
     </row>
-    <row r="31" spans="1:24" ht="28.5">
+    <row r="31" spans="1:24" ht="15">
       <c r="A31" s="1"/>
       <c r="B31" s="11"/>
       <c r="C31" s="3" t="s">
-        <v>55</v>
+        <v>14</v>
       </c>
       <c r="D31" s="1"/>
       <c r="E31" s="1"/>
@@ -2135,11 +2145,11 @@
       <c r="W31" s="1"/>
       <c r="X31" s="1"/>
     </row>
-    <row r="32" spans="1:24" ht="28.5">
+    <row r="32" spans="1:24" ht="15">
       <c r="A32" s="1"/>
       <c r="B32" s="11"/>
       <c r="C32" s="3" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="D32" s="1"/>
       <c r="E32" s="1"/>
@@ -2167,7 +2177,7 @@
       <c r="A33" s="1"/>
       <c r="B33" s="11"/>
       <c r="C33" s="3" t="s">
-        <v>21</v>
+        <v>55</v>
       </c>
       <c r="D33" s="1"/>
       <c r="E33" s="1"/>
@@ -2195,7 +2205,7 @@
       <c r="A34" s="1"/>
       <c r="B34" s="11"/>
       <c r="C34" s="3" t="s">
-        <v>47</v>
+        <v>20</v>
       </c>
       <c r="D34" s="1"/>
       <c r="E34" s="1"/>
@@ -2219,11 +2229,11 @@
       <c r="W34" s="1"/>
       <c r="X34" s="1"/>
     </row>
-    <row r="35" spans="1:24" ht="15">
+    <row r="35" spans="1:24" ht="28.5">
       <c r="A35" s="1"/>
       <c r="B35" s="11"/>
       <c r="C35" s="3" t="s">
-        <v>48</v>
+        <v>21</v>
       </c>
       <c r="D35" s="1"/>
       <c r="E35" s="1"/>
@@ -2247,11 +2257,11 @@
       <c r="W35" s="1"/>
       <c r="X35" s="1"/>
     </row>
-    <row r="36" spans="1:24" ht="15">
+    <row r="36" spans="1:24" ht="28.5">
       <c r="A36" s="1"/>
       <c r="B36" s="11"/>
       <c r="C36" s="3" t="s">
-        <v>0</v>
+        <v>47</v>
       </c>
       <c r="D36" s="1"/>
       <c r="E36" s="1"/>
@@ -2279,7 +2289,7 @@
       <c r="A37" s="1"/>
       <c r="B37" s="11"/>
       <c r="C37" s="3" t="s">
-        <v>1</v>
+        <v>48</v>
       </c>
       <c r="D37" s="1"/>
       <c r="E37" s="1"/>
@@ -2307,7 +2317,7 @@
       <c r="A38" s="1"/>
       <c r="B38" s="11"/>
       <c r="C38" s="3" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D38" s="1"/>
       <c r="E38" s="1"/>
@@ -2335,7 +2345,7 @@
       <c r="A39" s="1"/>
       <c r="B39" s="11"/>
       <c r="C39" s="3" t="s">
-        <v>34</v>
+        <v>1</v>
       </c>
       <c r="D39" s="1"/>
       <c r="E39" s="1"/>
@@ -2361,11 +2371,9 @@
     </row>
     <row r="40" spans="1:24" ht="15">
       <c r="A40" s="1"/>
-      <c r="B40" s="11" t="s">
-        <v>12</v>
-      </c>
+      <c r="B40" s="11"/>
       <c r="C40" s="3" t="s">
-        <v>50</v>
+        <v>2</v>
       </c>
       <c r="D40" s="1"/>
       <c r="E40" s="1"/>
@@ -2393,7 +2401,7 @@
       <c r="A41" s="1"/>
       <c r="B41" s="11"/>
       <c r="C41" s="3" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D41" s="1"/>
       <c r="E41" s="1"/>
@@ -2417,13 +2425,13 @@
       <c r="W41" s="1"/>
       <c r="X41" s="1"/>
     </row>
-    <row r="42" spans="1:24" ht="28.5">
+    <row r="42" spans="1:24" ht="15">
       <c r="A42" s="1"/>
       <c r="B42" s="11" t="s">
-        <v>49</v>
+        <v>12</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="D42" s="1"/>
       <c r="E42" s="1"/>
@@ -2451,7 +2459,7 @@
       <c r="A43" s="1"/>
       <c r="B43" s="11"/>
       <c r="C43" s="3" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D43" s="1"/>
       <c r="E43" s="1"/>
@@ -2475,13 +2483,13 @@
       <c r="W43" s="1"/>
       <c r="X43" s="1"/>
     </row>
-    <row r="44" spans="1:24" ht="15">
+    <row r="44" spans="1:24" ht="28.5">
       <c r="A44" s="1"/>
       <c r="B44" s="11" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>22</v>
+        <v>54</v>
       </c>
       <c r="D44" s="1"/>
       <c r="E44" s="1"/>
@@ -2509,7 +2517,7 @@
       <c r="A45" s="1"/>
       <c r="B45" s="11"/>
       <c r="C45" s="3" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D45" s="1"/>
       <c r="E45" s="1"/>
@@ -2536,10 +2544,10 @@
     <row r="46" spans="1:24" ht="15">
       <c r="A46" s="1"/>
       <c r="B46" s="11" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D46" s="1"/>
       <c r="E46" s="1"/>
@@ -2567,7 +2575,7 @@
       <c r="A47" s="1"/>
       <c r="B47" s="11"/>
       <c r="C47" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D47" s="1"/>
       <c r="E47" s="1"/>
@@ -2594,10 +2602,10 @@
     <row r="48" spans="1:24" ht="15">
       <c r="A48" s="1"/>
       <c r="B48" s="11" t="s">
-        <v>40</v>
+        <v>52</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>43</v>
+        <v>23</v>
       </c>
       <c r="D48" s="1"/>
       <c r="E48" s="1"/>
@@ -2625,7 +2633,7 @@
       <c r="A49" s="1"/>
       <c r="B49" s="11"/>
       <c r="C49" s="3" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="D49" s="1"/>
       <c r="E49" s="1"/>
@@ -2652,10 +2660,10 @@
     <row r="50" spans="1:24" ht="15">
       <c r="A50" s="1"/>
       <c r="B50" s="11" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D50" s="1"/>
       <c r="E50" s="1"/>
@@ -2683,7 +2691,7 @@
       <c r="A51" s="1"/>
       <c r="B51" s="11"/>
       <c r="C51" s="3" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D51" s="1"/>
       <c r="E51" s="1"/>
@@ -2710,10 +2718,10 @@
     <row r="52" spans="1:24" ht="15">
       <c r="A52" s="1"/>
       <c r="B52" s="11" t="s">
-        <v>13</v>
+        <v>41</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="D52" s="1"/>
       <c r="E52" s="1"/>
@@ -2737,10 +2745,12 @@
       <c r="W52" s="1"/>
       <c r="X52" s="1"/>
     </row>
-    <row r="53" spans="1:24">
+    <row r="53" spans="1:24" ht="15">
       <c r="A53" s="1"/>
-      <c r="B53" s="2"/>
-      <c r="C53" s="3"/>
+      <c r="B53" s="11"/>
+      <c r="C53" s="3" t="s">
+        <v>45</v>
+      </c>
       <c r="D53" s="1"/>
       <c r="E53" s="1"/>
       <c r="F53" s="1"/>
@@ -2763,8 +2773,14 @@
       <c r="W53" s="1"/>
       <c r="X53" s="1"/>
     </row>
-    <row r="54" spans="1:24">
+    <row r="54" spans="1:24" ht="15">
       <c r="A54" s="1"/>
+      <c r="B54" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="C54" s="3" t="s">
+        <v>39</v>
+      </c>
       <c r="D54" s="1"/>
       <c r="E54" s="1"/>
       <c r="F54" s="1"/>
@@ -2789,6 +2805,8 @@
     </row>
     <row r="55" spans="1:24">
       <c r="A55" s="1"/>
+      <c r="B55" s="2"/>
+      <c r="C55" s="3"/>
       <c r="D55" s="1"/>
       <c r="E55" s="1"/>
       <c r="F55" s="1"/>
@@ -2884,52 +2902,52 @@
       <c r="X58" s="1"/>
     </row>
     <row r="59" spans="1:24">
-      <c r="A59" s="12"/>
-      <c r="D59" s="12"/>
-      <c r="E59" s="12"/>
-      <c r="F59" s="12"/>
-      <c r="G59" s="12"/>
-      <c r="H59" s="12"/>
-      <c r="I59" s="12"/>
-      <c r="J59" s="12"/>
-      <c r="K59" s="12"/>
-      <c r="L59" s="12"/>
-      <c r="M59" s="12"/>
-      <c r="N59" s="12"/>
-      <c r="O59" s="12"/>
-      <c r="P59" s="12"/>
-      <c r="Q59" s="12"/>
-      <c r="R59" s="12"/>
-      <c r="S59" s="12"/>
-      <c r="T59" s="12"/>
-      <c r="U59" s="12"/>
-      <c r="V59" s="12"/>
-      <c r="W59" s="12"/>
-      <c r="X59" s="12"/>
+      <c r="A59" s="1"/>
+      <c r="D59" s="1"/>
+      <c r="E59" s="1"/>
+      <c r="F59" s="1"/>
+      <c r="G59" s="1"/>
+      <c r="H59" s="1"/>
+      <c r="I59" s="1"/>
+      <c r="J59" s="1"/>
+      <c r="K59" s="1"/>
+      <c r="L59" s="1"/>
+      <c r="M59" s="1"/>
+      <c r="N59" s="1"/>
+      <c r="O59" s="1"/>
+      <c r="P59" s="1"/>
+      <c r="Q59" s="1"/>
+      <c r="R59" s="1"/>
+      <c r="S59" s="1"/>
+      <c r="T59" s="1"/>
+      <c r="U59" s="1"/>
+      <c r="V59" s="1"/>
+      <c r="W59" s="1"/>
+      <c r="X59" s="1"/>
     </row>
     <row r="60" spans="1:24">
-      <c r="A60" s="12"/>
-      <c r="D60" s="12"/>
-      <c r="E60" s="12"/>
-      <c r="F60" s="12"/>
-      <c r="G60" s="12"/>
-      <c r="H60" s="12"/>
-      <c r="I60" s="12"/>
-      <c r="J60" s="12"/>
-      <c r="K60" s="12"/>
-      <c r="L60" s="12"/>
-      <c r="M60" s="12"/>
-      <c r="N60" s="12"/>
-      <c r="O60" s="12"/>
-      <c r="P60" s="12"/>
-      <c r="Q60" s="12"/>
-      <c r="R60" s="12"/>
-      <c r="S60" s="12"/>
-      <c r="T60" s="12"/>
-      <c r="U60" s="12"/>
-      <c r="V60" s="12"/>
-      <c r="W60" s="12"/>
-      <c r="X60" s="12"/>
+      <c r="A60" s="1"/>
+      <c r="D60" s="1"/>
+      <c r="E60" s="1"/>
+      <c r="F60" s="1"/>
+      <c r="G60" s="1"/>
+      <c r="H60" s="1"/>
+      <c r="I60" s="1"/>
+      <c r="J60" s="1"/>
+      <c r="K60" s="1"/>
+      <c r="L60" s="1"/>
+      <c r="M60" s="1"/>
+      <c r="N60" s="1"/>
+      <c r="O60" s="1"/>
+      <c r="P60" s="1"/>
+      <c r="Q60" s="1"/>
+      <c r="R60" s="1"/>
+      <c r="S60" s="1"/>
+      <c r="T60" s="1"/>
+      <c r="U60" s="1"/>
+      <c r="V60" s="1"/>
+      <c r="W60" s="1"/>
+      <c r="X60" s="1"/>
     </row>
     <row r="61" spans="1:24">
       <c r="A61" s="12"/>
@@ -3197,8 +3215,6 @@
     </row>
     <row r="72" spans="1:24">
       <c r="A72" s="12"/>
-      <c r="B72" s="7"/>
-      <c r="C72" s="13"/>
       <c r="D72" s="12"/>
       <c r="E72" s="12"/>
       <c r="F72" s="12"/>
@@ -3223,8 +3239,6 @@
     </row>
     <row r="73" spans="1:24">
       <c r="A73" s="12"/>
-      <c r="B73" s="7"/>
-      <c r="C73" s="13"/>
       <c r="D73" s="12"/>
       <c r="E73" s="12"/>
       <c r="F73" s="12"/>
@@ -8265,6 +8279,58 @@
       <c r="W266" s="12"/>
       <c r="X266" s="12"/>
     </row>
+    <row r="267" spans="1:24">
+      <c r="A267" s="12"/>
+      <c r="B267" s="7"/>
+      <c r="C267" s="13"/>
+      <c r="D267" s="12"/>
+      <c r="E267" s="12"/>
+      <c r="F267" s="12"/>
+      <c r="G267" s="12"/>
+      <c r="H267" s="12"/>
+      <c r="I267" s="12"/>
+      <c r="J267" s="12"/>
+      <c r="K267" s="12"/>
+      <c r="L267" s="12"/>
+      <c r="M267" s="12"/>
+      <c r="N267" s="12"/>
+      <c r="O267" s="12"/>
+      <c r="P267" s="12"/>
+      <c r="Q267" s="12"/>
+      <c r="R267" s="12"/>
+      <c r="S267" s="12"/>
+      <c r="T267" s="12"/>
+      <c r="U267" s="12"/>
+      <c r="V267" s="12"/>
+      <c r="W267" s="12"/>
+      <c r="X267" s="12"/>
+    </row>
+    <row r="268" spans="1:24">
+      <c r="A268" s="12"/>
+      <c r="B268" s="7"/>
+      <c r="C268" s="13"/>
+      <c r="D268" s="12"/>
+      <c r="E268" s="12"/>
+      <c r="F268" s="12"/>
+      <c r="G268" s="12"/>
+      <c r="H268" s="12"/>
+      <c r="I268" s="12"/>
+      <c r="J268" s="12"/>
+      <c r="K268" s="12"/>
+      <c r="L268" s="12"/>
+      <c r="M268" s="12"/>
+      <c r="N268" s="12"/>
+      <c r="O268" s="12"/>
+      <c r="P268" s="12"/>
+      <c r="Q268" s="12"/>
+      <c r="R268" s="12"/>
+      <c r="S268" s="12"/>
+      <c r="T268" s="12"/>
+      <c r="U268" s="12"/>
+      <c r="V268" s="12"/>
+      <c r="W268" s="12"/>
+      <c r="X268" s="12"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>